<commit_message>
v90: workout style Plan day cards, race standards on sim stations, Delson removed
Plan day cards now read like a workout card: weekday and date, a type tag (Strength, Running, Race sim, Hockey, Mobility, Recovery, Extra), the title, Est. minutes and exercise count (or results when logged), a big View workout button and a check square (filled when done, tap to log a past or current day). Sim station rows on Plan and Today show this week's distance and the HYROX race standard (distance and weight). Today: gap under the mobility card. Plan: removed the HSQ Delson tune up option from week 3 Saturday in PLAN and the Excel (Plan H4, Overview A62) at Fred's request.

Coach impact: week 3 Saturday plan text is now just the half sim (no Delson tune up option).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_017ty1gcaEfLM16MJZGfipS3
</commit_message>
<xml_diff>
--- a/plan/HYROX_Brisbane_2027_Plan.xlsx
+++ b/plan/HYROX_Brisbane_2027_Plan.xlsx
@@ -1464,11 +1464,7 @@
       </c>
     </row>
     <row r="62" ht="15" customHeight="1" s="39">
-      <c r="A62" s="42" t="inlineStr">
-        <is>
-          <t>• Optional tune up: HSQ half HYROX finale, Delson, Oct 17 to 18 2026 (week 3). Good baseline, not a target.</t>
-        </is>
-      </c>
+      <c r="A62" s="42" t="n"/>
     </row>
   </sheetData>
   <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0" gridLinesSet="1"/>
@@ -1707,7 +1703,7 @@
       </c>
       <c r="H4" s="49" t="inlineStr">
         <is>
-          <t>Tune up option: HSQ Delson Oct 17 to 18. Else half sim stations 1 to 4, half volume, 75%</t>
+          <t>Half sim stations 1 to 4, half volume, 75%</t>
         </is>
       </c>
       <c r="I4" s="49" t="inlineStr">
@@ -3008,7 +3004,6 @@
         </is>
       </c>
     </row>
-    <row r="29"/>
     <row r="30" ht="15" customHeight="1" s="39">
       <c r="A30" s="41" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
v98: overload block above race weight, clearer sled card
Plan (Fred asked on Oct 17): Monday EMOM farmers carries above race weight for grip (2 x 28 kg weeks 5 to 7, 2 x 32 kg over 60 m weeks 9 to 14, 2 x 30 kg over 100 m weeks 15 to 21); weeks 15 to 21 sled push and pull become 15 m at 110% race weight; lunges stay 20 kg; weeks 22+ and Saturday sims stay at race weight. PLAN and the Excel are updated. The sled suggestion cap follows the plan (110% of race weight on those Mondays only). Sled card now reads Suggested N lb total with the plates weight under it, and Plates + Empty sled = Total at the bottom.

Coach impact: PROMPT.md explains the overload block so the coach judges carries and sleds against the new plan loads. Log format unchanged.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_017ty1gcaEfLM16MJZGfipS3
</commit_message>
<xml_diff>
--- a/plan/HYROX_Brisbane_2027_Plan.xlsx
+++ b/plan/HYROX_Brisbane_2027_Plan.xlsx
@@ -1789,7 +1789,7 @@
       </c>
       <c r="E6" s="49" t="inlineStr">
         <is>
-          <t>Trap bar DL 3 x 5 heavy. Hack squat 3 x 8 @ RPE 7. EMOM 16 min (4 rounds), moderate: 1) sled push 20 m 2) 10 lunges/leg 10 kg 3) farmers carry 50 m, 2 x 24 kg 4) rest</t>
+          <t>Trap bar DL 3 x 5 heavy. Hack squat 3 x 8 @ RPE 7. EMOM 16 min (4 rounds), moderate: 1) sled push 20 m 2) 10 lunges/leg 10 kg 3) farmers carry 50 m, 2 x 28 kg (above race weight, grip) 4) rest</t>
         </is>
       </c>
       <c r="F6" s="49" t="inlineStr">
@@ -1841,7 +1841,7 @@
       </c>
       <c r="E7" s="49" t="inlineStr">
         <is>
-          <t>Trap bar DL 3 x 5 heavy. Hack squat 3 x 8 @ RPE 7. EMOM 16 min (4 rounds), moderate: 1) sled push 20 m (last round at race weight) 2) 10 lunges/leg 10 kg 3) farmers carry 50 m, 2 x 24 kg 4) rest</t>
+          <t>Trap bar DL 3 x 5 heavy. Hack squat 3 x 8 @ RPE 7. EMOM 16 min (4 rounds), moderate: 1) sled push 20 m (last round at race weight) 2) 10 lunges/leg 10 kg 3) farmers carry 50 m, 2 x 28 kg (above race weight, grip) 4) rest</t>
         </is>
       </c>
       <c r="F7" s="49" t="inlineStr">
@@ -1897,7 +1897,7 @@
       </c>
       <c r="E8" s="49" t="inlineStr">
         <is>
-          <t>Trap bar DL 3 x 5 heavy. Hack squat 3 x 8 @ RPE 7. EMOM 16 min (4 rounds), moderate: 1) sled push 20 m (last round at race weight) 2) 10 lunges/leg 10 kg 3) farmers carry 50 m, 2 x 24 kg 4) rest</t>
+          <t>Trap bar DL 3 x 5 heavy. Hack squat 3 x 8 @ RPE 7. EMOM 16 min (4 rounds), moderate: 1) sled push 20 m (last round at race weight) 2) 10 lunges/leg 10 kg 3) farmers carry 50 m, 2 x 28 kg (above race weight, grip) 4) rest</t>
         </is>
       </c>
       <c r="F8" s="49" t="inlineStr">
@@ -2005,7 +2005,7 @@
       </c>
       <c r="E10" s="49" t="inlineStr">
         <is>
-          <t>Back squat 3 x 5. RDL 3 x 8 @ RPE 7. EMOM 16 min (4 rounds, shorter: full sim Saturday): 1) sled push 25 m race weight 2) sandbag lunges 20 m, 20 kg 3) farmers 60 m race weight 4) sled pull 12.5 m race weight</t>
+          <t>Back squat 3 x 5. RDL 3 x 8 @ RPE 7. EMOM 16 min (4 rounds, shorter: full sim Saturday): 1) sled push 25 m race weight 2) sandbag lunges 20 m, 20 kg 3) farmers 60 m, 2 x 32 kg (above race weight, grip) 4) sled pull 12.5 m race weight</t>
         </is>
       </c>
       <c r="F10" s="49" t="inlineStr">
@@ -2061,7 +2061,7 @@
       </c>
       <c r="E11" s="49" t="inlineStr">
         <is>
-          <t>Back squat 3 x 5. RDL 3 x 8 @ RPE 7. EMOM 20 min (5 rounds): 1) sled push 25 m race weight 2) sandbag lunges 20 m, 20 kg 3) farmers 60 m race weight 4) sled pull 12.5 m race weight</t>
+          <t>Back squat 3 x 5. RDL 3 x 8 @ RPE 7. EMOM 20 min (5 rounds): 1) sled push 25 m race weight 2) sandbag lunges 20 m, 20 kg 3) farmers 60 m, 2 x 32 kg (above race weight, grip) 4) sled pull 12.5 m race weight</t>
         </is>
       </c>
       <c r="F11" s="49" t="inlineStr">
@@ -2113,7 +2113,7 @@
       </c>
       <c r="E12" s="49" t="inlineStr">
         <is>
-          <t>Back squat 3 x 5. RDL 3 x 8 @ RPE 7. EMOM 20 min (5 rounds): 1) sled push 25 m race weight 2) sandbag lunges 20 m, 20 kg 3) farmers 60 m race weight 4) sled pull 12.5 m race weight</t>
+          <t>Back squat 3 x 5. RDL 3 x 8 @ RPE 7. EMOM 20 min (5 rounds): 1) sled push 25 m race weight 2) sandbag lunges 20 m, 20 kg 3) farmers 60 m, 2 x 32 kg (above race weight, grip) 4) sled pull 12.5 m race weight</t>
         </is>
       </c>
       <c r="F12" s="49" t="inlineStr">
@@ -2221,7 +2221,7 @@
       </c>
       <c r="E14" s="49" t="inlineStr">
         <is>
-          <t>Back squat 3 x 5. RDL 3 x 8 @ RPE 7. EMOM 20 min (5 rounds): 1) sled push 25 m race weight 2) sandbag lunges 20 m, 20 kg 3) farmers 60 m race weight 4) sled pull 12.5 m race weight</t>
+          <t>Back squat 3 x 5. RDL 3 x 8 @ RPE 7. EMOM 20 min (5 rounds): 1) sled push 25 m race weight 2) sandbag lunges 20 m, 20 kg 3) farmers 60 m, 2 x 32 kg (above race weight, grip) 4) sled pull 12.5 m race weight</t>
         </is>
       </c>
       <c r="F14" s="49" t="inlineStr">
@@ -2277,7 +2277,7 @@
       </c>
       <c r="E15" s="49" t="inlineStr">
         <is>
-          <t>Back squat 3 x 5. RDL 3 x 8 @ RPE 7. EMOM 20 min (5 rounds): 1) sled push 25 m race weight 2) sandbag lunges 20 m, 20 kg 3) farmers 60 m race weight 4) sled pull 12.5 m race weight</t>
+          <t>Back squat 3 x 5. RDL 3 x 8 @ RPE 7. EMOM 20 min (5 rounds): 1) sled push 25 m race weight 2) sandbag lunges 20 m, 20 kg 3) farmers 60 m, 2 x 32 kg (above race weight, grip) 4) sled pull 12.5 m race weight</t>
         </is>
       </c>
       <c r="F15" s="49" t="inlineStr">
@@ -2329,7 +2329,7 @@
       </c>
       <c r="E16" s="49" t="inlineStr">
         <is>
-          <t>Back squat 3 x 5. RDL 3 x 8 @ RPE 7. EMOM 24 min, race weights: 1) sled push 25 m 2) sandbag lunges 25 m 3) farmers 100 m 4) sled pull 25 m above race weight</t>
+          <t>Back squat 3 x 5. RDL 3 x 8 @ RPE 7. EMOM 24 min: 1) sled push 15 m at 110% race weight 2) sandbag lunges 25 m, 20 kg 3) farmers 100 m, 2 x 30 kg (above race weight, grip) 4) sled pull 15 m at 110% race weight</t>
         </is>
       </c>
       <c r="F16" s="49" t="inlineStr">
@@ -2437,7 +2437,7 @@
       </c>
       <c r="E18" s="49" t="inlineStr">
         <is>
-          <t>Back squat 3 x 5. RDL 3 x 8 @ RPE 7. EMOM 24 min, race weights: 1) sled push 25 m 2) sandbag lunges 25 m 3) farmers 100 m 4) sled pull 25 m above race weight</t>
+          <t>Back squat 3 x 5. RDL 3 x 8 @ RPE 7. EMOM 24 min: 1) sled push 15 m at 110% race weight 2) sandbag lunges 25 m, 20 kg 3) farmers 100 m, 2 x 30 kg (above race weight, grip) 4) sled pull 15 m at 110% race weight</t>
         </is>
       </c>
       <c r="F18" s="49" t="inlineStr">
@@ -2489,7 +2489,7 @@
       </c>
       <c r="E19" s="49" t="inlineStr">
         <is>
-          <t>Back squat 3 x 5. RDL 3 x 8 @ RPE 7. EMOM 24 min, race weights: 1) sled push 25 m 2) sandbag lunges 25 m 3) farmers 100 m 4) sled pull 25 m above race weight</t>
+          <t>Back squat 3 x 5. RDL 3 x 8 @ RPE 7. EMOM 24 min: 1) sled push 15 m at 110% race weight 2) sandbag lunges 25 m, 20 kg 3) farmers 100 m, 2 x 30 kg (above race weight, grip) 4) sled pull 15 m at 110% race weight</t>
         </is>
       </c>
       <c r="F19" s="49" t="inlineStr">
@@ -2541,7 +2541,7 @@
       </c>
       <c r="E20" s="49" t="inlineStr">
         <is>
-          <t>Back squat 3 x 5. RDL 3 x 8 @ RPE 7. EMOM 16 min (shorter: full sim Saturday), race weights: 1) sled push 25 m 2) sandbag lunges 25 m 3) farmers 100 m 4) sled pull 25 m above race weight</t>
+          <t>Back squat 3 x 5. RDL 3 x 8 @ RPE 7. EMOM 16 min (shorter: full sim Saturday): 1) sled push 15 m at 110% race weight 2) sandbag lunges 25 m, 20 kg 3) farmers 100 m, 2 x 30 kg (above race weight, grip) 4) sled pull 15 m at 110% race weight</t>
         </is>
       </c>
       <c r="F20" s="49" t="inlineStr">
@@ -2653,7 +2653,7 @@
       </c>
       <c r="E22" s="49" t="inlineStr">
         <is>
-          <t>Back squat 3 x 5. RDL 3 x 8 @ RPE 7. EMOM 16 min (shorter: full sim Saturday), race weights: 1) sled push 25 m 2) sandbag lunges 25 m 3) farmers 100 m 4) sled pull 25 m above race weight</t>
+          <t>Back squat 3 x 5. RDL 3 x 8 @ RPE 7. EMOM 16 min (shorter: full sim Saturday): 1) sled push 15 m at 110% race weight 2) sandbag lunges 25 m, 20 kg 3) farmers 100 m, 2 x 30 kg (above race weight, grip) 4) sled pull 15 m at 110% race weight</t>
         </is>
       </c>
       <c r="F22" s="49" t="inlineStr">

</xml_diff>

<commit_message>
v103: Sunday easy run every week from week 3 to 25, run km targets updated
Fred agreed on Oct 18: he ran about half the planned km in weeks 1 to 3 and running is his biggest gap to 1:25. Sunday is now a planned easy run of 30 to 40 min at conversational pace (about 5 km), deload weeks included; week 25 is 30 min (taper) and week 11 stays optional after Nashville. runKm +5 per week (+4 in week 25). Sunday checks in the app accept the new text, so the run is loggable and shows as missed when skipped. PLAN and the Excel (Sunday and Run km columns) updated. Also fixed the grid, header and today85 tests for the v97 layout (#weekTrack, Today strip caption).

Coach impact: PROMPT.md explains the Sunday easy run and the new km targets; call out missed Tuesday and Sunday runs.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_017ty1gcaEfLM16MJZGfipS3
</commit_message>
<xml_diff>
--- a/plan/HYROX_Brisbane_2027_Plan.xlsx
+++ b/plan/HYROX_Brisbane_2027_Plan.xlsx
@@ -1538,7 +1538,7 @@
       </c>
       <c r="I1" s="48" t="inlineStr">
         <is>
-          <t>SUN: optional easy run</t>
+          <t>SUN: easy run</t>
         </is>
       </c>
       <c r="J1" s="48" t="inlineStr">
@@ -1708,11 +1708,11 @@
       </c>
       <c r="I4" s="49" t="inlineStr">
         <is>
-          <t>Rest</t>
+          <t>Easy run 30 to 40 min, conversational pace (about 5 km)</t>
         </is>
       </c>
       <c r="J4" s="49" t="n">
-        <v>9</v>
+        <v>14</v>
       </c>
       <c r="K4" s="58" t="n"/>
       <c r="L4" s="59" t="n"/>
@@ -1760,11 +1760,11 @@
       </c>
       <c r="I5" s="49" t="inlineStr">
         <is>
-          <t>Rest</t>
+          <t>Easy run 30 to 40 min, conversational pace (about 5 km)</t>
         </is>
       </c>
       <c r="J5" s="49" t="n">
-        <v>6</v>
+        <v>11</v>
       </c>
       <c r="K5" s="58" t="n"/>
       <c r="L5" s="59" t="n"/>
@@ -1812,11 +1812,11 @@
       </c>
       <c r="I6" s="49" t="inlineStr">
         <is>
-          <t>Rest</t>
+          <t>Easy run 30 to 40 min, conversational pace (about 5 km)</t>
         </is>
       </c>
       <c r="J6" s="49" t="n">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="K6" s="58" t="n"/>
       <c r="L6" s="59" t="n"/>
@@ -1864,11 +1864,11 @@
       </c>
       <c r="I7" s="49" t="inlineStr">
         <is>
-          <t>Rest</t>
+          <t>Easy run 30 to 40 min, conversational pace (about 5 km)</t>
         </is>
       </c>
       <c r="J7" s="49" t="n">
-        <v>11</v>
+        <v>16</v>
       </c>
       <c r="K7" s="58" t="n"/>
       <c r="L7" s="59" t="inlineStr">
@@ -1920,11 +1920,11 @@
       </c>
       <c r="I8" s="49" t="inlineStr">
         <is>
-          <t>Rest</t>
+          <t>Easy run 30 to 40 min, conversational pace (about 5 km)</t>
         </is>
       </c>
       <c r="J8" s="49" t="n">
-        <v>12</v>
+        <v>17</v>
       </c>
       <c r="K8" s="58" t="n"/>
       <c r="L8" s="59" t="n"/>
@@ -1972,11 +1972,11 @@
       </c>
       <c r="I9" s="49" t="inlineStr">
         <is>
-          <t>Rest</t>
+          <t>Easy run 30 to 40 min, conversational pace (about 5 km)</t>
         </is>
       </c>
       <c r="J9" s="49" t="n">
-        <v>8</v>
+        <v>13</v>
       </c>
       <c r="K9" s="58" t="n"/>
       <c r="L9" s="59" t="inlineStr">
@@ -2028,11 +2028,11 @@
       </c>
       <c r="I10" s="49" t="inlineStr">
         <is>
-          <t>Optional: 30 min easy, only if fresh</t>
+          <t>Easy run 30 to 40 min, conversational pace (about 5 km)</t>
         </is>
       </c>
       <c r="J10" s="49" t="n">
-        <v>12</v>
+        <v>17</v>
       </c>
       <c r="K10" s="58" t="n"/>
       <c r="L10" s="59" t="inlineStr">
@@ -2084,11 +2084,11 @@
       </c>
       <c r="I11" s="49" t="inlineStr">
         <is>
-          <t>Optional: 30 min easy, only if fresh</t>
+          <t>Easy run 30 to 40 min, conversational pace (about 5 km)</t>
         </is>
       </c>
       <c r="J11" s="49" t="n">
-        <v>13</v>
+        <v>18</v>
       </c>
       <c r="K11" s="58" t="n"/>
       <c r="L11" s="59" t="n"/>
@@ -2136,7 +2136,7 @@
       </c>
       <c r="I12" s="49" t="inlineStr">
         <is>
-          <t>Optional: 30 min easy, only if fresh</t>
+          <t>Optional: easy 20 to 30 min, only if fresh after the race</t>
         </is>
       </c>
       <c r="J12" s="49" t="n">
@@ -2192,11 +2192,11 @@
       </c>
       <c r="I13" s="49" t="inlineStr">
         <is>
-          <t>Rest</t>
+          <t>Easy run 30 to 40 min, conversational pace (about 5 km)</t>
         </is>
       </c>
       <c r="J13" s="49" t="n">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="K13" s="58" t="n"/>
       <c r="L13" s="59" t="n"/>
@@ -2244,11 +2244,11 @@
       </c>
       <c r="I14" s="49" t="inlineStr">
         <is>
-          <t>Optional: 30 min easy, only if fresh</t>
+          <t>Easy run 30 to 40 min, conversational pace (about 5 km)</t>
         </is>
       </c>
       <c r="J14" s="49" t="n">
-        <v>12</v>
+        <v>17</v>
       </c>
       <c r="K14" s="58" t="n"/>
       <c r="L14" s="59" t="inlineStr">
@@ -2300,11 +2300,11 @@
       </c>
       <c r="I15" s="49" t="inlineStr">
         <is>
-          <t>Optional: 30 min easy, only if fresh</t>
+          <t>Easy run 30 to 40 min, conversational pace (about 5 km)</t>
         </is>
       </c>
       <c r="J15" s="49" t="n">
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="K15" s="58" t="n"/>
       <c r="L15" s="59" t="n"/>
@@ -2352,11 +2352,11 @@
       </c>
       <c r="I16" s="49" t="inlineStr">
         <is>
-          <t>Optional: 30 min easy, only if fresh</t>
+          <t>Easy run 30 to 40 min, conversational pace (about 5 km)</t>
         </is>
       </c>
       <c r="J16" s="49" t="n">
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="K16" s="58" t="n"/>
       <c r="L16" s="59" t="n"/>
@@ -2404,11 +2404,11 @@
       </c>
       <c r="I17" s="49" t="inlineStr">
         <is>
-          <t>Rest</t>
+          <t>Easy run 30 to 40 min, conversational pace (about 5 km)</t>
         </is>
       </c>
       <c r="J17" s="49" t="n">
-        <v>11</v>
+        <v>16</v>
       </c>
       <c r="K17" s="58" t="n"/>
       <c r="L17" s="59" t="inlineStr">
@@ -2460,11 +2460,11 @@
       </c>
       <c r="I18" s="49" t="inlineStr">
         <is>
-          <t>Optional: 30 min easy, only if fresh</t>
+          <t>Easy run 30 to 40 min, conversational pace (about 5 km)</t>
         </is>
       </c>
       <c r="J18" s="49" t="n">
-        <v>16</v>
+        <v>21</v>
       </c>
       <c r="K18" s="58" t="n"/>
       <c r="L18" s="59" t="n"/>
@@ -2512,11 +2512,11 @@
       </c>
       <c r="I19" s="49" t="inlineStr">
         <is>
-          <t>Optional: 30 min easy, only if fresh</t>
+          <t>Easy run 30 to 40 min, conversational pace (about 5 km)</t>
         </is>
       </c>
       <c r="J19" s="49" t="n">
-        <v>17</v>
+        <v>22</v>
       </c>
       <c r="K19" s="58" t="n"/>
       <c r="L19" s="59" t="n"/>
@@ -2564,11 +2564,11 @@
       </c>
       <c r="I20" s="49" t="inlineStr">
         <is>
-          <t>Optional: 30 min easy, only if fresh</t>
+          <t>Easy run 30 to 40 min, conversational pace (about 5 km)</t>
         </is>
       </c>
       <c r="J20" s="49" t="n">
-        <v>18</v>
+        <v>23</v>
       </c>
       <c r="K20" s="58" t="n"/>
       <c r="L20" s="59" t="inlineStr">
@@ -2620,11 +2620,11 @@
       </c>
       <c r="I21" s="49" t="inlineStr">
         <is>
-          <t>Rest</t>
+          <t>Easy run 30 to 40 min, conversational pace (about 5 km)</t>
         </is>
       </c>
       <c r="J21" s="49" t="n">
-        <v>13</v>
+        <v>18</v>
       </c>
       <c r="K21" s="58" t="n"/>
       <c r="L21" s="59" t="inlineStr">
@@ -2676,11 +2676,11 @@
       </c>
       <c r="I22" s="49" t="inlineStr">
         <is>
-          <t>Optional: 30 min easy, only if fresh</t>
+          <t>Easy run 30 to 40 min, conversational pace (about 5 km)</t>
         </is>
       </c>
       <c r="J22" s="49" t="n">
-        <v>19</v>
+        <v>24</v>
       </c>
       <c r="K22" s="58" t="n"/>
       <c r="L22" s="59" t="n"/>
@@ -2728,11 +2728,11 @@
       </c>
       <c r="I23" s="49" t="inlineStr">
         <is>
-          <t>Optional: 30 min easy, only if fresh</t>
+          <t>Easy run 30 to 40 min, conversational pace (about 5 km)</t>
         </is>
       </c>
       <c r="J23" s="49" t="n">
-        <v>19</v>
+        <v>24</v>
       </c>
       <c r="K23" s="58" t="n"/>
       <c r="L23" s="59" t="n"/>
@@ -2780,11 +2780,11 @@
       </c>
       <c r="I24" s="49" t="inlineStr">
         <is>
-          <t>Optional: 30 min easy, only if fresh</t>
+          <t>Easy run 30 to 40 min, conversational pace (about 5 km)</t>
         </is>
       </c>
       <c r="J24" s="49" t="n">
-        <v>20</v>
+        <v>25</v>
       </c>
       <c r="K24" s="58" t="n"/>
       <c r="L24" s="59" t="n"/>
@@ -2832,11 +2832,11 @@
       </c>
       <c r="I25" s="49" t="inlineStr">
         <is>
-          <t>Optional: 30 min easy, only if fresh</t>
+          <t>Easy run 30 to 40 min, conversational pace (about 5 km)</t>
         </is>
       </c>
       <c r="J25" s="49" t="n">
-        <v>20</v>
+        <v>25</v>
       </c>
       <c r="K25" s="58" t="n"/>
       <c r="L25" s="59" t="inlineStr">
@@ -2888,11 +2888,11 @@
       </c>
       <c r="I26" s="49" t="inlineStr">
         <is>
-          <t>Rest</t>
+          <t>Easy run 30 min, conversational pace (taper)</t>
         </is>
       </c>
       <c r="J26" s="49" t="n">
-        <v>14</v>
+        <v>18</v>
       </c>
       <c r="K26" s="58" t="n"/>
       <c r="L26" s="59" t="n"/>

</xml_diff>

<commit_message>
v105: Sunday runs are zone 2 (130 to 140 bpm)
Fred asked to have zone 2 in the app. Sunday plan text for weeks 3 to 25 now reads Easy run 30 to 40 min in zone 2: 130 to 140 bpm, full sentences, slow is fine (about 5 km); taper and Nashville week variants too. The Plan Sunday card shows a Zone 2 · 130 to 140 bpm badge and the run detail explains the talk test. PLAN and the Excel updated.

Coach impact: PROMPT.md says Sunday runs are zone 2 at 130 to 140 bpm, and to track pace at the same heart rate.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_017ty1gcaEfLM16MJZGfipS3
</commit_message>
<xml_diff>
--- a/plan/HYROX_Brisbane_2027_Plan.xlsx
+++ b/plan/HYROX_Brisbane_2027_Plan.xlsx
@@ -1708,7 +1708,7 @@
       </c>
       <c r="I4" s="49" t="inlineStr">
         <is>
-          <t>Easy run 30 to 40 min, conversational pace (about 5 km)</t>
+          <t>Easy run 30 to 40 min in zone 2: 130 to 140 bpm, full sentences, slow is fine (about 5 km)</t>
         </is>
       </c>
       <c r="J4" s="49" t="n">
@@ -1760,7 +1760,7 @@
       </c>
       <c r="I5" s="49" t="inlineStr">
         <is>
-          <t>Easy run 30 to 40 min, conversational pace (about 5 km)</t>
+          <t>Easy run 30 to 40 min in zone 2: 130 to 140 bpm, full sentences, slow is fine (about 5 km)</t>
         </is>
       </c>
       <c r="J5" s="49" t="n">
@@ -1812,7 +1812,7 @@
       </c>
       <c r="I6" s="49" t="inlineStr">
         <is>
-          <t>Easy run 30 to 40 min, conversational pace (about 5 km)</t>
+          <t>Easy run 30 to 40 min in zone 2: 130 to 140 bpm, full sentences, slow is fine (about 5 km)</t>
         </is>
       </c>
       <c r="J6" s="49" t="n">
@@ -1864,7 +1864,7 @@
       </c>
       <c r="I7" s="49" t="inlineStr">
         <is>
-          <t>Easy run 30 to 40 min, conversational pace (about 5 km)</t>
+          <t>Easy run 30 to 40 min in zone 2: 130 to 140 bpm, full sentences, slow is fine (about 5 km)</t>
         </is>
       </c>
       <c r="J7" s="49" t="n">
@@ -1920,7 +1920,7 @@
       </c>
       <c r="I8" s="49" t="inlineStr">
         <is>
-          <t>Easy run 30 to 40 min, conversational pace (about 5 km)</t>
+          <t>Easy run 30 to 40 min in zone 2: 130 to 140 bpm, full sentences, slow is fine (about 5 km)</t>
         </is>
       </c>
       <c r="J8" s="49" t="n">
@@ -1972,7 +1972,7 @@
       </c>
       <c r="I9" s="49" t="inlineStr">
         <is>
-          <t>Easy run 30 to 40 min, conversational pace (about 5 km)</t>
+          <t>Easy run 30 to 40 min in zone 2: 130 to 140 bpm, full sentences, slow is fine (about 5 km)</t>
         </is>
       </c>
       <c r="J9" s="49" t="n">
@@ -2028,7 +2028,7 @@
       </c>
       <c r="I10" s="49" t="inlineStr">
         <is>
-          <t>Easy run 30 to 40 min, conversational pace (about 5 km)</t>
+          <t>Easy run 30 to 40 min in zone 2: 130 to 140 bpm, full sentences, slow is fine (about 5 km)</t>
         </is>
       </c>
       <c r="J10" s="49" t="n">
@@ -2084,7 +2084,7 @@
       </c>
       <c r="I11" s="49" t="inlineStr">
         <is>
-          <t>Easy run 30 to 40 min, conversational pace (about 5 km)</t>
+          <t>Easy run 30 to 40 min in zone 2: 130 to 140 bpm, full sentences, slow is fine (about 5 km)</t>
         </is>
       </c>
       <c r="J11" s="49" t="n">
@@ -2136,7 +2136,7 @@
       </c>
       <c r="I12" s="49" t="inlineStr">
         <is>
-          <t>Optional: easy 20 to 30 min, only if fresh after the race</t>
+          <t>Optional: easy 20 to 30 min in zone 2, only if fresh after the race</t>
         </is>
       </c>
       <c r="J12" s="49" t="n">
@@ -2192,7 +2192,7 @@
       </c>
       <c r="I13" s="49" t="inlineStr">
         <is>
-          <t>Easy run 30 to 40 min, conversational pace (about 5 km)</t>
+          <t>Easy run 30 to 40 min in zone 2: 130 to 140 bpm, full sentences, slow is fine (about 5 km)</t>
         </is>
       </c>
       <c r="J13" s="49" t="n">
@@ -2244,7 +2244,7 @@
       </c>
       <c r="I14" s="49" t="inlineStr">
         <is>
-          <t>Easy run 30 to 40 min, conversational pace (about 5 km)</t>
+          <t>Easy run 30 to 40 min in zone 2: 130 to 140 bpm, full sentences, slow is fine (about 5 km)</t>
         </is>
       </c>
       <c r="J14" s="49" t="n">
@@ -2300,7 +2300,7 @@
       </c>
       <c r="I15" s="49" t="inlineStr">
         <is>
-          <t>Easy run 30 to 40 min, conversational pace (about 5 km)</t>
+          <t>Easy run 30 to 40 min in zone 2: 130 to 140 bpm, full sentences, slow is fine (about 5 km)</t>
         </is>
       </c>
       <c r="J15" s="49" t="n">
@@ -2352,7 +2352,7 @@
       </c>
       <c r="I16" s="49" t="inlineStr">
         <is>
-          <t>Easy run 30 to 40 min, conversational pace (about 5 km)</t>
+          <t>Easy run 30 to 40 min in zone 2: 130 to 140 bpm, full sentences, slow is fine (about 5 km)</t>
         </is>
       </c>
       <c r="J16" s="49" t="n">
@@ -2404,7 +2404,7 @@
       </c>
       <c r="I17" s="49" t="inlineStr">
         <is>
-          <t>Easy run 30 to 40 min, conversational pace (about 5 km)</t>
+          <t>Easy run 30 to 40 min in zone 2: 130 to 140 bpm, full sentences, slow is fine (about 5 km)</t>
         </is>
       </c>
       <c r="J17" s="49" t="n">
@@ -2460,7 +2460,7 @@
       </c>
       <c r="I18" s="49" t="inlineStr">
         <is>
-          <t>Easy run 30 to 40 min, conversational pace (about 5 km)</t>
+          <t>Easy run 30 to 40 min in zone 2: 130 to 140 bpm, full sentences, slow is fine (about 5 km)</t>
         </is>
       </c>
       <c r="J18" s="49" t="n">
@@ -2512,7 +2512,7 @@
       </c>
       <c r="I19" s="49" t="inlineStr">
         <is>
-          <t>Easy run 30 to 40 min, conversational pace (about 5 km)</t>
+          <t>Easy run 30 to 40 min in zone 2: 130 to 140 bpm, full sentences, slow is fine (about 5 km)</t>
         </is>
       </c>
       <c r="J19" s="49" t="n">
@@ -2564,7 +2564,7 @@
       </c>
       <c r="I20" s="49" t="inlineStr">
         <is>
-          <t>Easy run 30 to 40 min, conversational pace (about 5 km)</t>
+          <t>Easy run 30 to 40 min in zone 2: 130 to 140 bpm, full sentences, slow is fine (about 5 km)</t>
         </is>
       </c>
       <c r="J20" s="49" t="n">
@@ -2620,7 +2620,7 @@
       </c>
       <c r="I21" s="49" t="inlineStr">
         <is>
-          <t>Easy run 30 to 40 min, conversational pace (about 5 km)</t>
+          <t>Easy run 30 to 40 min in zone 2: 130 to 140 bpm, full sentences, slow is fine (about 5 km)</t>
         </is>
       </c>
       <c r="J21" s="49" t="n">
@@ -2676,7 +2676,7 @@
       </c>
       <c r="I22" s="49" t="inlineStr">
         <is>
-          <t>Easy run 30 to 40 min, conversational pace (about 5 km)</t>
+          <t>Easy run 30 to 40 min in zone 2: 130 to 140 bpm, full sentences, slow is fine (about 5 km)</t>
         </is>
       </c>
       <c r="J22" s="49" t="n">
@@ -2728,7 +2728,7 @@
       </c>
       <c r="I23" s="49" t="inlineStr">
         <is>
-          <t>Easy run 30 to 40 min, conversational pace (about 5 km)</t>
+          <t>Easy run 30 to 40 min in zone 2: 130 to 140 bpm, full sentences, slow is fine (about 5 km)</t>
         </is>
       </c>
       <c r="J23" s="49" t="n">
@@ -2780,7 +2780,7 @@
       </c>
       <c r="I24" s="49" t="inlineStr">
         <is>
-          <t>Easy run 30 to 40 min, conversational pace (about 5 km)</t>
+          <t>Easy run 30 to 40 min in zone 2: 130 to 140 bpm, full sentences, slow is fine (about 5 km)</t>
         </is>
       </c>
       <c r="J24" s="49" t="n">
@@ -2832,7 +2832,7 @@
       </c>
       <c r="I25" s="49" t="inlineStr">
         <is>
-          <t>Easy run 30 to 40 min, conversational pace (about 5 km)</t>
+          <t>Easy run 30 to 40 min in zone 2: 130 to 140 bpm, full sentences, slow is fine (about 5 km)</t>
         </is>
       </c>
       <c r="J25" s="49" t="n">
@@ -2888,7 +2888,7 @@
       </c>
       <c r="I26" s="49" t="inlineStr">
         <is>
-          <t>Easy run 30 min, conversational pace (taper)</t>
+          <t>Easy run 30 min in zone 2: 130 to 140 bpm (taper)</t>
         </is>
       </c>
       <c r="J26" s="49" t="n">

</xml_diff>

<commit_message>
v107: deload weeks cut volume, keep intensity
Fred (Oct 19): the old deload cut weights, sets and reps at once and was too easy.
Weeks 4, 8, 12, 16, 20 now: lifts 3 sets @ 80% of last normal load, EMOM 12 min
(3 rounds) at normal loads, Tuesday 4 intervals at normal pace, arms 3 sets each,
Saturday sim 75%. Run km +1 (wk 4), +2 (wk 8).

App: "@ 80%" shows as an "80% of last" chip; suggestLoad keeps 80% for lifts but
EMOM moves and sleds hold the last load in deload weeks; lastLoad skips deload week
logs so the next normal week builds from the week before the deload (this also
fixes the week after a deload starting from the 80% loads). Excel Plan rows and
Overview deload line updated. Test: tests/deload.js, tests/sled.js updated.

Coach impact: PROMPT.md explains the new deload and says not to read deload
loads as a regression.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_017ty1gcaEfLM16MJZGfipS3
</commit_message>
<xml_diff>
--- a/plan/HYROX_Brisbane_2027_Plan.xlsx
+++ b/plan/HYROX_Brisbane_2027_Plan.xlsx
@@ -1424,7 +1424,7 @@
     <row r="56" ht="15" customHeight="1" s="39">
       <c r="A56" s="42" t="inlineStr">
         <is>
-          <t>• Weeks 4, 8, 12, 16, 20 are deloads: main lift 2 sets, secondary leg lift 2 x 8 light, EMOM 12 min light, about 30% less volume overall.</t>
+          <t>• Weeks 4, 8, 12, 16, 20 are deloads (changed Oct 19): lifts 3 sets at 80% of last load, EMOM 12 min at normal loads, Tuesday 4 intervals at normal pace, arms 3 sets each, Saturday sim at 75%. Volume drops, intensity stays.</t>
         </is>
       </c>
     </row>
@@ -1737,25 +1737,25 @@
       </c>
       <c r="E5" s="49" t="inlineStr">
         <is>
-          <t>Main lift 2 x 5 light. Hack squat 2 x 8 light. EMOM 12 min light (3 rounds): 1) sled push 20 m 2) 10 lunges/leg 3) farmers 50 m 4) rest</t>
+          <t>Trap bar DL 3 x 5 @ 80%. Hack squat 3 x 8 @ 80%. EMOM 12 min (3 rounds), normal loads: 1) sled push 20 m 2) 10 lunges/leg bodyweight 3) farmers carry 50 m, 2 x 24 kg 4) rest</t>
         </is>
       </c>
       <c r="F5" s="49" t="inlineStr">
         <is>
-          <t>4 x 400 m easy
-Then arms block A, 2 sets each: Lateral raises 4x12-15, incline DB curls 3x10, overhead triceps ext 3x10, hanging leg raises 3x10-12</t>
+          <t>4 x 600 m, 90 s rest
+Then arms block A, 3 sets each: Lateral raises 3x12-15, incline DB curls 3x10, overhead triceps ext 3x10, hanging leg raises 3x10-12</t>
         </is>
       </c>
       <c r="G5" s="49" t="inlineStr">
         <is>
-          <t>Pull ups 2 x 5, press 2 x 5.
-Then arms block B, 2 sets each: Face pulls 3x15, cable crunch 3x10
-Finisher: EMOM 12 min light: 1) SkiErg 125 m 2) 15 wall balls 3) row 125 m 4) rest</t>
+          <t>Weighted pull ups 3 x 5 @ 80%, DB bench 3 x 8 @ 80%.
+Then arms block B: Face pulls 3x15, cable crunch 3x10
+Finisher: EMOM 12 min: 1) SkiErg 150 m 2) 15 wall balls 3) row 150 m 4) rest</t>
         </is>
       </c>
       <c r="H5" s="49" t="inlineStr">
         <is>
-          <t>Half sim, 70%, half volume, stations 1 to 4</t>
+          <t>Half sim, 75%, half volume, stations 1 to 4</t>
         </is>
       </c>
       <c r="I5" s="49" t="inlineStr">
@@ -1764,7 +1764,7 @@
         </is>
       </c>
       <c r="J5" s="49" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="K5" s="58" t="n"/>
       <c r="L5" s="59" t="n"/>
@@ -1949,25 +1949,25 @@
       </c>
       <c r="E9" s="49" t="inlineStr">
         <is>
-          <t>Main lift 2 x 5 light. Hack squat 2 x 8 light. EMOM 12 min light (3 rounds): 1) sled push 20 m 2) 10 lunges/leg 3) farmers 50 m 4) rest</t>
+          <t>Trap bar DL 3 x 5 @ 80%. Hack squat 3 x 8 @ 80%. EMOM 12 min (3 rounds), normal loads: 1) sled push 20 m 2) 10 lunges/leg 10 kg 3) farmers carry 50 m, 2 x 28 kg (above race weight, grip) 4) rest</t>
         </is>
       </c>
       <c r="F9" s="49" t="inlineStr">
         <is>
-          <t>4 x 400 m easy
-Then arms block A, 2 sets each: Lateral raises 4x12-15, incline DB curls 3x10, overhead triceps ext 3x10, hanging leg raises 3x10-12</t>
+          <t>4 x 1 km @ 10k pace, 2 min rest
+Then arms block A, 3 sets each: Lateral raises 3x12-15, incline DB curls 3x10, overhead triceps ext 3x10, hanging leg raises 3x10-12</t>
         </is>
       </c>
       <c r="G9" s="49" t="inlineStr">
         <is>
-          <t>Pull ups 2 x 5, press 2 x 5.
-Then arms block B, 2 sets each: Face pulls 3x15, cable crunch 3x10
-Finisher: EMOM 12 min light: 1) SkiErg 125 m 2) 15 wall balls 3) row 125 m 4) rest</t>
+          <t>Weighted pull ups 3 x 5 @ 80%, DB bench 3 x 8 @ 80%.
+Then arms block B: Face pulls 3x15, cable crunch 3x10
+Finisher: EMOM 12 min: 1) SkiErg 150 m 2) 15 wall balls 3) row 150 m 4) rest</t>
         </is>
       </c>
       <c r="H9" s="49" t="inlineStr">
         <is>
-          <t>Half sim, 70%, half volume, stations 5 to 8</t>
+          <t>Half sim, 75%, half volume, stations 5 to 8</t>
         </is>
       </c>
       <c r="I9" s="49" t="inlineStr">
@@ -1976,7 +1976,7 @@
         </is>
       </c>
       <c r="J9" s="49" t="n">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="K9" s="58" t="n"/>
       <c r="L9" s="59" t="inlineStr">
@@ -2169,25 +2169,25 @@
       </c>
       <c r="E13" s="49" t="inlineStr">
         <is>
-          <t>Main lift 2 x 5 light. RDL 2 x 8 light. EMOM 12 min light (3 rounds): 1) sled push 20 m 2) 10 lunges/leg 3) farmers 50 m 4) rest</t>
+          <t>Back squat 3 x 5 @ 80%. RDL 3 x 8 @ 80%. EMOM 12 min (3 rounds), normal loads: 1) sled push 25 m race weight 2) sandbag lunges 20 m, 20 kg 3) farmers 60 m, 2 x 32 kg (above race weight, grip) 4) sled pull 12.5 m race weight</t>
         </is>
       </c>
       <c r="F13" s="49" t="inlineStr">
         <is>
-          <t>5 x 1 km easy
-Then arms block A, 2 sets each: Lateral raises 4x12-15, incline DB curls 3x10, overhead triceps ext 3x10, hanging leg raises 3x10-12</t>
+          <t>4 x 1 km @ race pace, 2 min rest
+Then arms block A, 3 sets each: Lateral raises 3x12-15, incline DB curls 3x10, overhead triceps ext 3x10, hanging leg raises 3x10-12</t>
         </is>
       </c>
       <c r="G13" s="49" t="inlineStr">
         <is>
-          <t>Pull ups 2 x 5, press 2 x 5.
-Then arms block B, 2 sets each: Face pulls 3x15, cable crunch 3x10
-Finisher: EMOM 12 min light: 1) SkiErg 125 m 2) 15 wall balls 3) row 125 m 4) rest</t>
+          <t>Weighted pull ups 3 x 5 @ 80%, OHP 3 x 5 @ 80%.
+Then arms block B: Face pulls 3x15, cable crunch 3x10
+Finisher: EMOM 12 min: 1) SkiErg 200 m 2) 20 wall balls 3) 8 burpee broad jumps 4) row 200 m</t>
         </is>
       </c>
       <c r="H13" s="49" t="inlineStr">
         <is>
-          <t>Half sim, 70%, half volume, stations 5 to 8</t>
+          <t>Half sim, 75%, half volume, stations 5 to 8</t>
         </is>
       </c>
       <c r="I13" s="49" t="inlineStr">
@@ -2381,25 +2381,25 @@
       </c>
       <c r="E17" s="49" t="inlineStr">
         <is>
-          <t>Main lift 2 x 5 light. RDL 2 x 8 light. EMOM 12 min light (3 rounds): 1) sled push 20 m 2) 10 lunges/leg 3) farmers 50 m 4) rest</t>
+          <t>Back squat 3 x 5 @ 80%. RDL 3 x 8 @ 80%. EMOM 12 min (3 rounds), normal loads: 1) sled push 15 m at 110% race weight 2) sandbag lunges 25 m, 20 kg 3) farmers 100 m, 2 x 30 kg (above race weight, grip) 4) sled pull 15 m at 110% race weight</t>
         </is>
       </c>
       <c r="F17" s="49" t="inlineStr">
         <is>
-          <t>5 x 1 km easy
-Then arms block A, 2 sets each: Lateral raises 4x12-15, incline DB curls 3x10, overhead triceps ext 3x10, hanging leg raises 3x10-12</t>
+          <t>4 x 1 km @ race pace, 90 s rest
+Then arms block A, 3 sets each: Lateral raises 3x12-15, incline DB curls 3x10, overhead triceps ext 3x10, hanging leg raises 3x10-12</t>
         </is>
       </c>
       <c r="G17" s="49" t="inlineStr">
         <is>
-          <t>Pull ups 2 x 5, press 2 x 5.
-Then arms block B, 2 sets each: Face pulls 3x15, cable crunch 3x10
-Finisher: EMOM 12 min light: 1) SkiErg 125 m 2) 15 wall balls 3) row 125 m 4) rest</t>
+          <t>Weighted pull ups 3 x 5 @ 80%, bench 3 x 5 @ 80%.
+Then arms block B: Face pulls 3x15, cable crunch 3x10
+Finisher: EMOM 12 min: 1) SkiErg 250 m 2) 25 wall balls 3) 10 burpee broad jumps 4) row 250 m</t>
         </is>
       </c>
       <c r="H17" s="49" t="inlineStr">
         <is>
-          <t>Half sim, 70%, stations 1 to 4 full volume</t>
+          <t>Half sim, 75%, stations 1 to 4 full volume</t>
         </is>
       </c>
       <c r="I17" s="49" t="inlineStr">
@@ -2597,25 +2597,25 @@
       </c>
       <c r="E21" s="49" t="inlineStr">
         <is>
-          <t>Main lift 2 x 5 light. RDL 2 x 8 light. EMOM 12 min light (3 rounds): 1) sled push 20 m 2) 10 lunges/leg 3) farmers 50 m 4) rest</t>
+          <t>Back squat 3 x 5 @ 80%. RDL 3 x 8 @ 80%. EMOM 12 min (3 rounds), normal loads: 1) sled push 15 m at 110% race weight 2) sandbag lunges 25 m, 20 kg 3) farmers 100 m, 2 x 30 kg (above race weight, grip) 4) sled pull 15 m at 110% race weight</t>
         </is>
       </c>
       <c r="F21" s="49" t="inlineStr">
         <is>
-          <t>5 x 1 km easy
-Then arms block A, 2 sets each: Lateral raises 4x12-15, incline DB curls 3x10, overhead triceps ext 3x10, hanging leg raises 3x10-12</t>
+          <t>4 x 1 km @ race pace, 90 s rest
+Then arms block A, 3 sets each: Lateral raises 3x12-15, incline DB curls 3x10, overhead triceps ext 3x10, hanging leg raises 3x10-12</t>
         </is>
       </c>
       <c r="G21" s="49" t="inlineStr">
         <is>
-          <t>Pull ups 2 x 5, press 2 x 5.
-Then arms block B, 2 sets each: Face pulls 3x15, cable crunch 3x10
-Finisher: EMOM 12 min light: 1) SkiErg 125 m 2) 15 wall balls 3) row 125 m 4) rest</t>
+          <t>Weighted pull ups 3 x 5 @ 80%, bench 3 x 5 @ 80%.
+Then arms block B: Face pulls 3x15, cable crunch 3x10
+Finisher: EMOM 12 min: 1) SkiErg 250 m 2) 25 wall balls 3) 10 burpee broad jumps 4) row 250 m</t>
         </is>
       </c>
       <c r="H21" s="49" t="inlineStr">
         <is>
-          <t>Half sim, 70%, stations 5 to 8 full volume</t>
+          <t>Half sim, 75%, stations 5 to 8 full volume</t>
         </is>
       </c>
       <c r="I21" s="49" t="inlineStr">
@@ -3004,6 +3004,7 @@
         </is>
       </c>
     </row>
+    <row r="29"/>
     <row r="30" ht="15" customHeight="1" s="39">
       <c r="A30" s="41" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
v111: biceps block (about 10 direct sets a week)
Fred (Oct 20): his biceps have not grown in years. Plan change he approved:
Tue incline DB curls 4x8-12 (3x8-12 in deloads) for weeks 5 to 24; Fri arms
block B adds Bayesian cable curls 3x10-12 and hammer curls 3x10-12 for weeks
4 to 24. History (weeks 1 to 3) and taper (25 to 27) unchanged. New guide
bayescurl (matcher, increment, rest, video query). Friday card reads 6 lifts
+ EMOM. Excel Plan columns F and G updated. Test: tests/biceps.js.

Coach impact: PROMPT.md explains the biceps block, the new Loads names
(Bayesian cable curl, Hammer curl) and to track the three curl loads.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_017ty1gcaEfLM16MJZGfipS3
</commit_message>
<xml_diff>
--- a/plan/HYROX_Brisbane_2027_Plan.xlsx
+++ b/plan/HYROX_Brisbane_2027_Plan.xlsx
@@ -1749,7 +1749,7 @@
       <c r="G5" s="49" t="inlineStr">
         <is>
           <t>Weighted pull ups 3 x 5 @ 80%, DB bench 3 x 8 @ 80%.
-Then arms block B: Face pulls 3x15, cable crunch 3x10
+Then arms block B: Face pulls 3x15, Bayesian cable curls 3x10-12, hammer curls 3x10-12, cable crunch 3x10
 Finisher: EMOM 12 min: 1) SkiErg 150 m 2) 15 wall balls 3) row 150 m 4) rest</t>
         </is>
       </c>
@@ -1795,13 +1795,13 @@
       <c r="F6" s="49" t="inlineStr">
         <is>
           <t>4 x 1 km @ 10k pace, 2 min rest
-Then arms block A: Lateral raises 4x12-15, incline DB curls 3x10, overhead triceps ext 3x10, hanging leg raises 3x10-12</t>
+Then arms block A: Lateral raises 4x12-15, incline DB curls 4x8-12, overhead triceps ext 3x10, hanging leg raises 3x10-12</t>
         </is>
       </c>
       <c r="G6" s="49" t="inlineStr">
         <is>
           <t>Weighted pull ups 3 x 5, DB bench 3 x 8.
-Then arms block B: Face pulls 3x15, cable crunch 3x10
+Then arms block B: Face pulls 3x15, Bayesian cable curls 3x10-12, hammer curls 3x10-12, cable crunch 3x10
 Finisher: EMOM 16 min: 1) SkiErg 150 m 2) 15 wall balls 3) row 150 m 4) rest</t>
         </is>
       </c>
@@ -1847,13 +1847,13 @@
       <c r="F7" s="49" t="inlineStr">
         <is>
           <t>5 x 1 km @ 10k pace, 2 min rest
-Then arms block A: Lateral raises 4x12-15, incline DB curls 3x10, overhead triceps ext 3x10, hanging leg raises 3x10-12</t>
+Then arms block A: Lateral raises 4x12-15, incline DB curls 4x8-12, overhead triceps ext 3x10, hanging leg raises 3x10-12</t>
         </is>
       </c>
       <c r="G7" s="49" t="inlineStr">
         <is>
           <t>Weighted pull ups 3 x 5, DB bench 3 x 8.
-Then arms block B: Face pulls 3x15, cable crunch 3x10
+Then arms block B: Face pulls 3x15, Bayesian cable curls 3x10-12, hammer curls 3x10-12, cable crunch 3x10
 Finisher: EMOM 16 min: 1) SkiErg 150 m 2) 15 wall balls 3) row 150 m 4) rest</t>
         </is>
       </c>
@@ -1903,13 +1903,13 @@
       <c r="F8" s="49" t="inlineStr">
         <is>
           <t>5 x 1 km @ 10k pace, 90 s rest
-Then arms block A: Lateral raises 4x12-15, incline DB curls 3x10, overhead triceps ext 3x10, hanging leg raises 3x10-12</t>
+Then arms block A: Lateral raises 4x12-15, incline DB curls 4x8-12, overhead triceps ext 3x10, hanging leg raises 3x10-12</t>
         </is>
       </c>
       <c r="G8" s="49" t="inlineStr">
         <is>
           <t>Weighted pull ups 3 x 5, DB bench 3 x 8.
-Then arms block B: Face pulls 3x15, cable crunch 3x10
+Then arms block B: Face pulls 3x15, Bayesian cable curls 3x10-12, hammer curls 3x10-12, cable crunch 3x10
 Finisher: EMOM 16 min: 1) SkiErg 150 m 2) 15 wall balls 3) row 150 m 4) rest</t>
         </is>
       </c>
@@ -1955,13 +1955,13 @@
       <c r="F9" s="49" t="inlineStr">
         <is>
           <t>4 x 1 km @ 10k pace, 2 min rest
-Then arms block A, 3 sets each: Lateral raises 3x12-15, incline DB curls 3x10, overhead triceps ext 3x10, hanging leg raises 3x10-12</t>
+Then arms block A, 3 sets each: Lateral raises 3x12-15, incline DB curls 3x8-12, overhead triceps ext 3x10, hanging leg raises 3x10-12</t>
         </is>
       </c>
       <c r="G9" s="49" t="inlineStr">
         <is>
           <t>Weighted pull ups 3 x 5 @ 80%, DB bench 3 x 8 @ 80%.
-Then arms block B: Face pulls 3x15, cable crunch 3x10
+Then arms block B: Face pulls 3x15, Bayesian cable curls 3x10-12, hammer curls 3x10-12, cable crunch 3x10
 Finisher: EMOM 12 min: 1) SkiErg 150 m 2) 15 wall balls 3) row 150 m 4) rest</t>
         </is>
       </c>
@@ -2011,13 +2011,13 @@
       <c r="F10" s="49" t="inlineStr">
         <is>
           <t>6 x 1 km @ race pace, 90 s rest
-Then arms block A: Lateral raises 4x12-15, incline DB curls 3x10, overhead triceps ext 3x10, hanging leg raises 3x10-12</t>
+Then arms block A: Lateral raises 4x12-15, incline DB curls 4x8-12, overhead triceps ext 3x10, hanging leg raises 3x10-12</t>
         </is>
       </c>
       <c r="G10" s="49" t="inlineStr">
         <is>
           <t>Weighted pull ups 3 x 5, OHP 3 x 5.
-Then arms block B: Face pulls 3x15, cable crunch 3x10
+Then arms block B: Face pulls 3x15, Bayesian cable curls 3x10-12, hammer curls 3x10-12, cable crunch 3x10
 Finisher: EMOM 20 min: 1) SkiErg 200 m 2) 20 wall balls 3) 8 burpee broad jumps 4) row 200 m</t>
         </is>
       </c>
@@ -2067,13 +2067,13 @@
       <c r="F11" s="49" t="inlineStr">
         <is>
           <t>6 x 1 km @ race pace, 75 s rest
-Then arms block A: Lateral raises 4x12-15, incline DB curls 3x10, overhead triceps ext 3x10, hanging leg raises 3x10-12</t>
+Then arms block A: Lateral raises 4x12-15, incline DB curls 4x8-12, overhead triceps ext 3x10, hanging leg raises 3x10-12</t>
         </is>
       </c>
       <c r="G11" s="49" t="inlineStr">
         <is>
           <t>Weighted pull ups 3 x 5, OHP 3 x 5.
-Then arms block B: Face pulls 3x15, cable crunch 3x10
+Then arms block B: Face pulls 3x15, Bayesian cable curls 3x10-12, hammer curls 3x10-12, cable crunch 3x10
 Finisher: EMOM 20 min: 1) SkiErg 200 m 2) 20 wall balls 3) 8 burpee broad jumps 4) row 200 m</t>
         </is>
       </c>
@@ -2119,13 +2119,13 @@
       <c r="F12" s="49" t="inlineStr">
         <is>
           <t>3 x 2 km @ race pace, 2 min rest
-Then arms block A: Lateral raises 4x12-15, incline DB curls 3x10, overhead triceps ext 3x10, hanging leg raises 3x10-12</t>
+Then arms block A: Lateral raises 4x12-15, incline DB curls 4x8-12, overhead triceps ext 3x10, hanging leg raises 3x10-12</t>
         </is>
       </c>
       <c r="G12" s="49" t="inlineStr">
         <is>
           <t>Weighted pull ups 3 x 5, OHP 3 x 5.
-Then arms block B: Face pulls 3x15, cable crunch 3x10
+Then arms block B: Face pulls 3x15, Bayesian cable curls 3x10-12, hammer curls 3x10-12, cable crunch 3x10
 Finisher: EMOM 20 min: 1) SkiErg 200 m 2) 20 wall balls 3) 8 burpee broad jumps 4) row 200 m</t>
         </is>
       </c>
@@ -2175,13 +2175,13 @@
       <c r="F13" s="49" t="inlineStr">
         <is>
           <t>4 x 1 km @ race pace, 2 min rest
-Then arms block A, 3 sets each: Lateral raises 3x12-15, incline DB curls 3x10, overhead triceps ext 3x10, hanging leg raises 3x10-12</t>
+Then arms block A, 3 sets each: Lateral raises 3x12-15, incline DB curls 3x8-12, overhead triceps ext 3x10, hanging leg raises 3x10-12</t>
         </is>
       </c>
       <c r="G13" s="49" t="inlineStr">
         <is>
           <t>Weighted pull ups 3 x 5 @ 80%, OHP 3 x 5 @ 80%.
-Then arms block B: Face pulls 3x15, cable crunch 3x10
+Then arms block B: Face pulls 3x15, Bayesian cable curls 3x10-12, hammer curls 3x10-12, cable crunch 3x10
 Finisher: EMOM 12 min: 1) SkiErg 200 m 2) 20 wall balls 3) 8 burpee broad jumps 4) row 200 m</t>
         </is>
       </c>
@@ -2227,13 +2227,13 @@
       <c r="F14" s="49" t="inlineStr">
         <is>
           <t>Holiday week: 5 km tempo
-Then arms block A: Lateral raises 4x12-15, incline DB curls 3x10, overhead triceps ext 3x10, hanging leg raises 3x10-12</t>
+Then arms block A: Lateral raises 4x12-15, incline DB curls 4x8-12, overhead triceps ext 3x10, hanging leg raises 3x10-12</t>
         </is>
       </c>
       <c r="G14" s="49" t="inlineStr">
         <is>
           <t>Weighted pull ups 3 x 5, OHP 3 x 5.
-Then arms block B: Face pulls 3x15, cable crunch 3x10
+Then arms block B: Face pulls 3x15, Bayesian cable curls 3x10-12, hammer curls 3x10-12, cable crunch 3x10
 Finisher: EMOM 20 min: 1) SkiErg 200 m 2) 25 wall balls 3) 8 burpee broad jumps 4) row 200 m</t>
         </is>
       </c>
@@ -2283,13 +2283,13 @@
       <c r="F15" s="49" t="inlineStr">
         <is>
           <t>8 x 1 km @ race pace, 60 s rest
-Then arms block A: Lateral raises 4x12-15, incline DB curls 3x10, overhead triceps ext 3x10, hanging leg raises 3x10-12</t>
+Then arms block A: Lateral raises 4x12-15, incline DB curls 4x8-12, overhead triceps ext 3x10, hanging leg raises 3x10-12</t>
         </is>
       </c>
       <c r="G15" s="49" t="inlineStr">
         <is>
           <t>Weighted pull ups 3 x 5, OHP 3 x 5.
-Then arms block B: Face pulls 3x15, cable crunch 3x10
+Then arms block B: Face pulls 3x15, Bayesian cable curls 3x10-12, hammer curls 3x10-12, cable crunch 3x10
 Finisher: EMOM 20 min: 1) SkiErg 200 m 2) 25 wall balls 3) 8 burpee broad jumps 4) row 200 m</t>
         </is>
       </c>
@@ -2335,13 +2335,13 @@
       <c r="F16" s="49" t="inlineStr">
         <is>
           <t>5 km tempo @ slightly faster than race pace
-Then arms block A: Lateral raises 4x12-15, incline DB curls 3x10, overhead triceps ext 3x10, hanging leg raises 3x10-12</t>
+Then arms block A: Lateral raises 4x12-15, incline DB curls 4x8-12, overhead triceps ext 3x10, hanging leg raises 3x10-12</t>
         </is>
       </c>
       <c r="G16" s="49" t="inlineStr">
         <is>
           <t>Weighted pull ups 3 x 5, bench 3 x 5.
-Then arms block B: Face pulls 3x15, cable crunch 3x10
+Then arms block B: Face pulls 3x15, Bayesian cable curls 3x10-12, hammer curls 3x10-12, cable crunch 3x10
 Finisher: EMOM 24 min: 1) SkiErg 250 m 2) 25 wall balls 3) 10 burpee broad jumps 4) row 250 m</t>
         </is>
       </c>
@@ -2387,13 +2387,13 @@
       <c r="F17" s="49" t="inlineStr">
         <is>
           <t>4 x 1 km @ race pace, 90 s rest
-Then arms block A, 3 sets each: Lateral raises 3x12-15, incline DB curls 3x10, overhead triceps ext 3x10, hanging leg raises 3x10-12</t>
+Then arms block A, 3 sets each: Lateral raises 3x12-15, incline DB curls 3x8-12, overhead triceps ext 3x10, hanging leg raises 3x10-12</t>
         </is>
       </c>
       <c r="G17" s="49" t="inlineStr">
         <is>
           <t>Weighted pull ups 3 x 5 @ 80%, bench 3 x 5 @ 80%.
-Then arms block B: Face pulls 3x15, cable crunch 3x10
+Then arms block B: Face pulls 3x15, Bayesian cable curls 3x10-12, hammer curls 3x10-12, cable crunch 3x10
 Finisher: EMOM 12 min: 1) SkiErg 250 m 2) 25 wall balls 3) 10 burpee broad jumps 4) row 250 m</t>
         </is>
       </c>
@@ -2443,13 +2443,13 @@
       <c r="F18" s="49" t="inlineStr">
         <is>
           <t>4 x 2 km @ race pace, 90 s rest
-Then arms block A: Lateral raises 4x12-15, incline DB curls 3x10, overhead triceps ext 3x10, hanging leg raises 3x10-12</t>
+Then arms block A: Lateral raises 4x12-15, incline DB curls 4x8-12, overhead triceps ext 3x10, hanging leg raises 3x10-12</t>
         </is>
       </c>
       <c r="G18" s="49" t="inlineStr">
         <is>
           <t>Weighted pull ups 3 x 5, bench 3 x 5.
-Then arms block B: Face pulls 3x15, cable crunch 3x10
+Then arms block B: Face pulls 3x15, Bayesian cable curls 3x10-12, hammer curls 3x10-12, cable crunch 3x10
 Finisher: EMOM 24 min: 1) SkiErg 250 m 2) 25 wall balls 3) 10 burpee broad jumps 4) row 250 m</t>
         </is>
       </c>
@@ -2495,13 +2495,13 @@
       <c r="F19" s="49" t="inlineStr">
         <is>
           <t>6 km tempo
-Then arms block A: Lateral raises 4x12-15, incline DB curls 3x10, overhead triceps ext 3x10, hanging leg raises 3x10-12</t>
+Then arms block A: Lateral raises 4x12-15, incline DB curls 4x8-12, overhead triceps ext 3x10, hanging leg raises 3x10-12</t>
         </is>
       </c>
       <c r="G19" s="49" t="inlineStr">
         <is>
           <t>Weighted pull ups 3 x 5, bench 3 x 5.
-Then arms block B: Face pulls 3x15, cable crunch 3x10
+Then arms block B: Face pulls 3x15, Bayesian cable curls 3x10-12, hammer curls 3x10-12, cable crunch 3x10
 Finisher: EMOM 24 min: 1) SkiErg 250 m 2) 25 wall balls 3) 10 burpee broad jumps 4) row 250 m</t>
         </is>
       </c>
@@ -2547,13 +2547,13 @@
       <c r="F20" s="49" t="inlineStr">
         <is>
           <t>Easy 5 km (full sim Saturday)
-Then arms block A: Lateral raises 4x12-15, incline DB curls 3x10, overhead triceps ext 3x10, hanging leg raises 3x10-12</t>
+Then arms block A: Lateral raises 4x12-15, incline DB curls 4x8-12, overhead triceps ext 3x10, hanging leg raises 3x10-12</t>
         </is>
       </c>
       <c r="G20" s="49" t="inlineStr">
         <is>
           <t>Weighted pull ups 3 x 5, bench 3 x 5.
-Then arms block B: Face pulls 3x15, cable crunch 3x10
+Then arms block B: Face pulls 3x15, Bayesian cable curls 3x10-12, hammer curls 3x10-12, cable crunch 3x10
 Finisher: EMOM 16 min (shorter: full sim Saturday): 1) SkiErg 250 m 2) 25 wall balls 3) 10 burpee broad jumps 4) row 250 m</t>
         </is>
       </c>
@@ -2603,13 +2603,13 @@
       <c r="F21" s="49" t="inlineStr">
         <is>
           <t>4 x 1 km @ race pace, 90 s rest
-Then arms block A, 3 sets each: Lateral raises 3x12-15, incline DB curls 3x10, overhead triceps ext 3x10, hanging leg raises 3x10-12</t>
+Then arms block A, 3 sets each: Lateral raises 3x12-15, incline DB curls 3x8-12, overhead triceps ext 3x10, hanging leg raises 3x10-12</t>
         </is>
       </c>
       <c r="G21" s="49" t="inlineStr">
         <is>
           <t>Weighted pull ups 3 x 5 @ 80%, bench 3 x 5 @ 80%.
-Then arms block B: Face pulls 3x15, cable crunch 3x10
+Then arms block B: Face pulls 3x15, Bayesian cable curls 3x10-12, hammer curls 3x10-12, cable crunch 3x10
 Finisher: EMOM 12 min: 1) SkiErg 250 m 2) 25 wall balls 3) 10 burpee broad jumps 4) row 250 m</t>
         </is>
       </c>
@@ -2659,13 +2659,13 @@
       <c r="F22" s="49" t="inlineStr">
         <is>
           <t>3 x 3 km @ race pace, 2 min rest
-Then arms block A: Lateral raises 4x12-15, incline DB curls 3x10, overhead triceps ext 3x10, hanging leg raises 3x10-12</t>
+Then arms block A: Lateral raises 4x12-15, incline DB curls 4x8-12, overhead triceps ext 3x10, hanging leg raises 3x10-12</t>
         </is>
       </c>
       <c r="G22" s="49" t="inlineStr">
         <is>
           <t>Weighted pull ups 3 x 5, bench 3 x 5.
-Then arms block B: Face pulls 3x15, cable crunch 3x10
+Then arms block B: Face pulls 3x15, Bayesian cable curls 3x10-12, hammer curls 3x10-12, cable crunch 3x10
 Finisher: EMOM 16 min (shorter: full sim Saturday): 1) SkiErg 250 m 2) 25 wall balls 3) 10 burpee broad jumps 4) row 250 m</t>
         </is>
       </c>
@@ -2711,13 +2711,13 @@
       <c r="F23" s="49" t="inlineStr">
         <is>
           <t>6 x 1 km @ race pace, 60 s rest
-Then arms block A: Lateral raises 4x12-15, incline DB curls 3x10, overhead triceps ext 3x10, hanging leg raises 3x10-12</t>
+Then arms block A: Lateral raises 4x12-15, incline DB curls 4x8-12, overhead triceps ext 3x10, hanging leg raises 3x10-12</t>
         </is>
       </c>
       <c r="G23" s="49" t="inlineStr">
         <is>
           <t>Pull ups 3 x 5, press 3 x 5.
-Then arms block B: Face pulls 3x15, cable crunch 3x10
+Then arms block B: Face pulls 3x15, Bayesian cable curls 3x10-12, hammer curls 3x10-12, cable crunch 3x10
 Finisher: EMOM 20 min at race effort: 1) SkiErg 250 m 2) 25 wall balls 3) 10 burpee broad jumps 4) row 250 m</t>
         </is>
       </c>
@@ -2763,13 +2763,13 @@
       <c r="F24" s="49" t="inlineStr">
         <is>
           <t>8 x 1 km @ race pace, 45 s rest
-Then arms block A: Lateral raises 4x12-15, incline DB curls 3x10, overhead triceps ext 3x10, hanging leg raises 3x10-12</t>
+Then arms block A: Lateral raises 4x12-15, incline DB curls 4x8-12, overhead triceps ext 3x10, hanging leg raises 3x10-12</t>
         </is>
       </c>
       <c r="G24" s="49" t="inlineStr">
         <is>
           <t>Pull ups 3 x 5, press 3 x 5.
-Then arms block B: Face pulls 3x15, cable crunch 3x10
+Then arms block B: Face pulls 3x15, Bayesian cable curls 3x10-12, hammer curls 3x10-12, cable crunch 3x10
 Finisher: EMOM 20 min at race effort: 1) SkiErg 250 m 2) 25 wall balls 3) 10 burpee broad jumps 4) row 250 m</t>
         </is>
       </c>
@@ -2815,13 +2815,13 @@
       <c r="F25" s="49" t="inlineStr">
         <is>
           <t>Easy 5 km (dress rehearsal Saturday)
-Then arms block A: Lateral raises 4x12-15, incline DB curls 3x10, overhead triceps ext 3x10, hanging leg raises 3x10-12</t>
+Then arms block A: Lateral raises 4x12-15, incline DB curls 4x8-12, overhead triceps ext 3x10, hanging leg raises 3x10-12</t>
         </is>
       </c>
       <c r="G25" s="49" t="inlineStr">
         <is>
           <t>Pull ups 2 x 5.
-Then arms block B: Face pulls 3x15, cable crunch 3x10
+Then arms block B: Face pulls 3x15, Bayesian cable curls 3x10-12, hammer curls 3x10-12, cable crunch 3x10
 Finisher: EMOM 8 min light: SkiErg, wall balls, row, rest</t>
         </is>
       </c>
@@ -3004,7 +3004,6 @@
         </is>
       </c>
     </row>
-    <row r="29"/>
     <row r="30" ht="15" customHeight="1" s="39">
       <c r="A30" s="41" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
v113: move cable crunch from Friday to Monday (weeks 5 to 23)
Fred (Oct 23): Friday felt like too many exercises and Monday too few.
Cable crunch 3x10 moves from Friday arms block B to Monday, before the
EMOM. Friday is now pull ups, press, face pulls, Bayesian curls, hammer
curls, then the EMOM. Fred does not want extra leg work on Monday.
Badges follow the crunch (Mon Legs + Core, Fri Upper + Arms). Excel E
and G updated. Test: tests/balance.js.

Coach impact: PROMPT.md notes the move and that Monday gets no extra leg
exercises.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_017ty1gcaEfLM16MJZGfipS3
</commit_message>
<xml_diff>
--- a/plan/HYROX_Brisbane_2027_Plan.xlsx
+++ b/plan/HYROX_Brisbane_2027_Plan.xlsx
@@ -1789,7 +1789,7 @@
       </c>
       <c r="E6" s="49" t="inlineStr">
         <is>
-          <t>Trap bar DL 3 x 5 heavy. Hack squat 3 x 8 @ RPE 7. EMOM 16 min (4 rounds), moderate: 1) sled push 20 m 2) 10 lunges/leg 10 kg 3) farmers carry 50 m, 2 x 28 kg (above race weight, grip) 4) rest</t>
+          <t>Trap bar DL 3 x 5 heavy. Hack squat 3 x 8 @ RPE 7. Cable crunch 3x10. EMOM 16 min (4 rounds), moderate: 1) sled push 20 m 2) 10 lunges/leg 10 kg 3) farmers carry 50 m, 2 x 28 kg (above race weight, grip) 4) rest</t>
         </is>
       </c>
       <c r="F6" s="49" t="inlineStr">
@@ -1801,7 +1801,7 @@
       <c r="G6" s="49" t="inlineStr">
         <is>
           <t>Weighted pull ups 3 x 5, DB bench 3 x 8.
-Then arms block B: Face pulls 3x15, Bayesian cable curls 3x10-12, hammer curls 3x10-12, cable crunch 3x10
+Then arms block B: Face pulls 3x15, Bayesian cable curls 3x10-12, hammer curls 3x10-12
 Finisher: EMOM 16 min: 1) SkiErg 150 m 2) 15 wall balls 3) row 150 m 4) rest</t>
         </is>
       </c>
@@ -1841,7 +1841,7 @@
       </c>
       <c r="E7" s="49" t="inlineStr">
         <is>
-          <t>Trap bar DL 3 x 5 heavy. Hack squat 3 x 8 @ RPE 7. EMOM 16 min (4 rounds), moderate: 1) sled push 20 m (last round at race weight) 2) 10 lunges/leg 10 kg 3) farmers carry 50 m, 2 x 28 kg (above race weight, grip) 4) rest</t>
+          <t>Trap bar DL 3 x 5 heavy. Hack squat 3 x 8 @ RPE 7. Cable crunch 3x10. EMOM 16 min (4 rounds), moderate: 1) sled push 20 m (last round at race weight) 2) 10 lunges/leg 10 kg 3) farmers carry 50 m, 2 x 28 kg (above race weight, grip) 4) rest</t>
         </is>
       </c>
       <c r="F7" s="49" t="inlineStr">
@@ -1853,7 +1853,7 @@
       <c r="G7" s="49" t="inlineStr">
         <is>
           <t>Weighted pull ups 3 x 5, DB bench 3 x 8.
-Then arms block B: Face pulls 3x15, Bayesian cable curls 3x10-12, hammer curls 3x10-12, cable crunch 3x10
+Then arms block B: Face pulls 3x15, Bayesian cable curls 3x10-12, hammer curls 3x10-12
 Finisher: EMOM 16 min: 1) SkiErg 150 m 2) 15 wall balls 3) row 150 m 4) rest</t>
         </is>
       </c>
@@ -1897,7 +1897,7 @@
       </c>
       <c r="E8" s="49" t="inlineStr">
         <is>
-          <t>Trap bar DL 3 x 5 heavy. Hack squat 3 x 8 @ RPE 7. EMOM 16 min (4 rounds), moderate: 1) sled push 20 m (last round at race weight) 2) 10 lunges/leg 10 kg 3) farmers carry 50 m, 2 x 28 kg (above race weight, grip) 4) rest</t>
+          <t>Trap bar DL 3 x 5 heavy. Hack squat 3 x 8 @ RPE 7. Cable crunch 3x10. EMOM 16 min (4 rounds), moderate: 1) sled push 20 m (last round at race weight) 2) 10 lunges/leg 10 kg 3) farmers carry 50 m, 2 x 28 kg (above race weight, grip) 4) rest</t>
         </is>
       </c>
       <c r="F8" s="49" t="inlineStr">
@@ -1909,7 +1909,7 @@
       <c r="G8" s="49" t="inlineStr">
         <is>
           <t>Weighted pull ups 3 x 5, DB bench 3 x 8.
-Then arms block B: Face pulls 3x15, Bayesian cable curls 3x10-12, hammer curls 3x10-12, cable crunch 3x10
+Then arms block B: Face pulls 3x15, Bayesian cable curls 3x10-12, hammer curls 3x10-12
 Finisher: EMOM 16 min: 1) SkiErg 150 m 2) 15 wall balls 3) row 150 m 4) rest</t>
         </is>
       </c>
@@ -1949,7 +1949,7 @@
       </c>
       <c r="E9" s="49" t="inlineStr">
         <is>
-          <t>Trap bar DL 3 x 5 @ 80%. Hack squat 3 x 8 @ 80%. EMOM 12 min (3 rounds), normal loads: 1) sled push 20 m 2) 10 lunges/leg 10 kg 3) farmers carry 50 m, 2 x 28 kg (above race weight, grip) 4) rest</t>
+          <t>Trap bar DL 3 x 5 @ 80%. Hack squat 3 x 8 @ 80%. Cable crunch 3x10. EMOM 12 min (3 rounds), normal loads: 1) sled push 20 m 2) 10 lunges/leg 10 kg 3) farmers carry 50 m, 2 x 28 kg (above race weight, grip) 4) rest</t>
         </is>
       </c>
       <c r="F9" s="49" t="inlineStr">
@@ -1961,7 +1961,7 @@
       <c r="G9" s="49" t="inlineStr">
         <is>
           <t>Weighted pull ups 3 x 5 @ 80%, DB bench 3 x 8 @ 80%.
-Then arms block B: Face pulls 3x15, Bayesian cable curls 3x10-12, hammer curls 3x10-12, cable crunch 3x10
+Then arms block B: Face pulls 3x15, Bayesian cable curls 3x10-12, hammer curls 3x10-12
 Finisher: EMOM 12 min: 1) SkiErg 150 m 2) 15 wall balls 3) row 150 m 4) rest</t>
         </is>
       </c>
@@ -2005,7 +2005,7 @@
       </c>
       <c r="E10" s="49" t="inlineStr">
         <is>
-          <t>Back squat 3 x 5. RDL 3 x 8 @ RPE 7. EMOM 16 min (4 rounds, shorter: full sim Saturday): 1) sled push 25 m race weight 2) sandbag lunges 20 m, 20 kg 3) farmers 60 m, 2 x 32 kg (above race weight, grip) 4) sled pull 12.5 m race weight</t>
+          <t>Back squat 3 x 5. RDL 3 x 8 @ RPE 7. Cable crunch 3x10. EMOM 16 min (4 rounds, shorter: full sim Saturday): 1) sled push 25 m race weight 2) sandbag lunges 20 m, 20 kg 3) farmers 60 m, 2 x 32 kg (above race weight, grip) 4) sled pull 12.5 m race weight</t>
         </is>
       </c>
       <c r="F10" s="49" t="inlineStr">
@@ -2017,7 +2017,7 @@
       <c r="G10" s="49" t="inlineStr">
         <is>
           <t>Weighted pull ups 3 x 5, OHP 3 x 5.
-Then arms block B: Face pulls 3x15, Bayesian cable curls 3x10-12, hammer curls 3x10-12, cable crunch 3x10
+Then arms block B: Face pulls 3x15, Bayesian cable curls 3x10-12, hammer curls 3x10-12
 Finisher: EMOM 20 min: 1) SkiErg 200 m 2) 20 wall balls 3) 8 burpee broad jumps 4) row 200 m</t>
         </is>
       </c>
@@ -2061,7 +2061,7 @@
       </c>
       <c r="E11" s="49" t="inlineStr">
         <is>
-          <t>Back squat 3 x 5. RDL 3 x 8 @ RPE 7. EMOM 20 min (5 rounds): 1) sled push 25 m race weight 2) sandbag lunges 20 m, 20 kg 3) farmers 60 m, 2 x 32 kg (above race weight, grip) 4) sled pull 12.5 m race weight</t>
+          <t>Back squat 3 x 5. RDL 3 x 8 @ RPE 7. Cable crunch 3x10. EMOM 20 min (5 rounds): 1) sled push 25 m race weight 2) sandbag lunges 20 m, 20 kg 3) farmers 60 m, 2 x 32 kg (above race weight, grip) 4) sled pull 12.5 m race weight</t>
         </is>
       </c>
       <c r="F11" s="49" t="inlineStr">
@@ -2073,7 +2073,7 @@
       <c r="G11" s="49" t="inlineStr">
         <is>
           <t>Weighted pull ups 3 x 5, OHP 3 x 5.
-Then arms block B: Face pulls 3x15, Bayesian cable curls 3x10-12, hammer curls 3x10-12, cable crunch 3x10
+Then arms block B: Face pulls 3x15, Bayesian cable curls 3x10-12, hammer curls 3x10-12
 Finisher: EMOM 20 min: 1) SkiErg 200 m 2) 20 wall balls 3) 8 burpee broad jumps 4) row 200 m</t>
         </is>
       </c>
@@ -2113,7 +2113,7 @@
       </c>
       <c r="E12" s="49" t="inlineStr">
         <is>
-          <t>Back squat 3 x 5. RDL 3 x 8 @ RPE 7. EMOM 20 min (5 rounds): 1) sled push 25 m race weight 2) sandbag lunges 20 m, 20 kg 3) farmers 60 m, 2 x 32 kg (above race weight, grip) 4) sled pull 12.5 m race weight</t>
+          <t>Back squat 3 x 5. RDL 3 x 8 @ RPE 7. Cable crunch 3x10. EMOM 20 min (5 rounds): 1) sled push 25 m race weight 2) sandbag lunges 20 m, 20 kg 3) farmers 60 m, 2 x 32 kg (above race weight, grip) 4) sled pull 12.5 m race weight</t>
         </is>
       </c>
       <c r="F12" s="49" t="inlineStr">
@@ -2125,7 +2125,7 @@
       <c r="G12" s="49" t="inlineStr">
         <is>
           <t>Weighted pull ups 3 x 5, OHP 3 x 5.
-Then arms block B: Face pulls 3x15, Bayesian cable curls 3x10-12, hammer curls 3x10-12, cable crunch 3x10
+Then arms block B: Face pulls 3x15, Bayesian cable curls 3x10-12, hammer curls 3x10-12
 Finisher: EMOM 20 min: 1) SkiErg 200 m 2) 20 wall balls 3) 8 burpee broad jumps 4) row 200 m</t>
         </is>
       </c>
@@ -2169,7 +2169,7 @@
       </c>
       <c r="E13" s="49" t="inlineStr">
         <is>
-          <t>Back squat 3 x 5 @ 80%. RDL 3 x 8 @ 80%. EMOM 12 min (3 rounds), normal loads: 1) sled push 25 m race weight 2) sandbag lunges 20 m, 20 kg 3) farmers 60 m, 2 x 32 kg (above race weight, grip) 4) sled pull 12.5 m race weight</t>
+          <t>Back squat 3 x 5 @ 80%. RDL 3 x 8 @ 80%. Cable crunch 3x10. EMOM 12 min (3 rounds), normal loads: 1) sled push 25 m race weight 2) sandbag lunges 20 m, 20 kg 3) farmers 60 m, 2 x 32 kg (above race weight, grip) 4) sled pull 12.5 m race weight</t>
         </is>
       </c>
       <c r="F13" s="49" t="inlineStr">
@@ -2181,7 +2181,7 @@
       <c r="G13" s="49" t="inlineStr">
         <is>
           <t>Weighted pull ups 3 x 5 @ 80%, OHP 3 x 5 @ 80%.
-Then arms block B: Face pulls 3x15, Bayesian cable curls 3x10-12, hammer curls 3x10-12, cable crunch 3x10
+Then arms block B: Face pulls 3x15, Bayesian cable curls 3x10-12, hammer curls 3x10-12
 Finisher: EMOM 12 min: 1) SkiErg 200 m 2) 20 wall balls 3) 8 burpee broad jumps 4) row 200 m</t>
         </is>
       </c>
@@ -2221,7 +2221,7 @@
       </c>
       <c r="E14" s="49" t="inlineStr">
         <is>
-          <t>Back squat 3 x 5. RDL 3 x 8 @ RPE 7. EMOM 20 min (5 rounds): 1) sled push 25 m race weight 2) sandbag lunges 20 m, 20 kg 3) farmers 60 m, 2 x 32 kg (above race weight, grip) 4) sled pull 12.5 m race weight</t>
+          <t>Back squat 3 x 5. RDL 3 x 8 @ RPE 7. Cable crunch 3x10. EMOM 20 min (5 rounds): 1) sled push 25 m race weight 2) sandbag lunges 20 m, 20 kg 3) farmers 60 m, 2 x 32 kg (above race weight, grip) 4) sled pull 12.5 m race weight</t>
         </is>
       </c>
       <c r="F14" s="49" t="inlineStr">
@@ -2233,7 +2233,7 @@
       <c r="G14" s="49" t="inlineStr">
         <is>
           <t>Weighted pull ups 3 x 5, OHP 3 x 5.
-Then arms block B: Face pulls 3x15, Bayesian cable curls 3x10-12, hammer curls 3x10-12, cable crunch 3x10
+Then arms block B: Face pulls 3x15, Bayesian cable curls 3x10-12, hammer curls 3x10-12
 Finisher: EMOM 20 min: 1) SkiErg 200 m 2) 25 wall balls 3) 8 burpee broad jumps 4) row 200 m</t>
         </is>
       </c>
@@ -2277,7 +2277,7 @@
       </c>
       <c r="E15" s="49" t="inlineStr">
         <is>
-          <t>Back squat 3 x 5. RDL 3 x 8 @ RPE 7. EMOM 20 min (5 rounds): 1) sled push 25 m race weight 2) sandbag lunges 20 m, 20 kg 3) farmers 60 m, 2 x 32 kg (above race weight, grip) 4) sled pull 12.5 m race weight</t>
+          <t>Back squat 3 x 5. RDL 3 x 8 @ RPE 7. Cable crunch 3x10. EMOM 20 min (5 rounds): 1) sled push 25 m race weight 2) sandbag lunges 20 m, 20 kg 3) farmers 60 m, 2 x 32 kg (above race weight, grip) 4) sled pull 12.5 m race weight</t>
         </is>
       </c>
       <c r="F15" s="49" t="inlineStr">
@@ -2289,7 +2289,7 @@
       <c r="G15" s="49" t="inlineStr">
         <is>
           <t>Weighted pull ups 3 x 5, OHP 3 x 5.
-Then arms block B: Face pulls 3x15, Bayesian cable curls 3x10-12, hammer curls 3x10-12, cable crunch 3x10
+Then arms block B: Face pulls 3x15, Bayesian cable curls 3x10-12, hammer curls 3x10-12
 Finisher: EMOM 20 min: 1) SkiErg 200 m 2) 25 wall balls 3) 8 burpee broad jumps 4) row 200 m</t>
         </is>
       </c>
@@ -2329,7 +2329,7 @@
       </c>
       <c r="E16" s="49" t="inlineStr">
         <is>
-          <t>Back squat 3 x 5. RDL 3 x 8 @ RPE 7. EMOM 24 min: 1) sled push 15 m at 110% race weight 2) sandbag lunges 25 m, 20 kg 3) farmers 100 m, 2 x 30 kg (above race weight, grip) 4) sled pull 15 m at 110% race weight</t>
+          <t>Back squat 3 x 5. RDL 3 x 8 @ RPE 7. Cable crunch 3x10. EMOM 24 min: 1) sled push 15 m at 110% race weight 2) sandbag lunges 25 m, 20 kg 3) farmers 100 m, 2 x 30 kg (above race weight, grip) 4) sled pull 15 m at 110% race weight</t>
         </is>
       </c>
       <c r="F16" s="49" t="inlineStr">
@@ -2341,7 +2341,7 @@
       <c r="G16" s="49" t="inlineStr">
         <is>
           <t>Weighted pull ups 3 x 5, bench 3 x 5.
-Then arms block B: Face pulls 3x15, Bayesian cable curls 3x10-12, hammer curls 3x10-12, cable crunch 3x10
+Then arms block B: Face pulls 3x15, Bayesian cable curls 3x10-12, hammer curls 3x10-12
 Finisher: EMOM 24 min: 1) SkiErg 250 m 2) 25 wall balls 3) 10 burpee broad jumps 4) row 250 m</t>
         </is>
       </c>
@@ -2381,7 +2381,7 @@
       </c>
       <c r="E17" s="49" t="inlineStr">
         <is>
-          <t>Back squat 3 x 5 @ 80%. RDL 3 x 8 @ 80%. EMOM 12 min (3 rounds), normal loads: 1) sled push 15 m at 110% race weight 2) sandbag lunges 25 m, 20 kg 3) farmers 100 m, 2 x 30 kg (above race weight, grip) 4) sled pull 15 m at 110% race weight</t>
+          <t>Back squat 3 x 5 @ 80%. RDL 3 x 8 @ 80%. Cable crunch 3x10. EMOM 12 min (3 rounds), normal loads: 1) sled push 15 m at 110% race weight 2) sandbag lunges 25 m, 20 kg 3) farmers 100 m, 2 x 30 kg (above race weight, grip) 4) sled pull 15 m at 110% race weight</t>
         </is>
       </c>
       <c r="F17" s="49" t="inlineStr">
@@ -2393,7 +2393,7 @@
       <c r="G17" s="49" t="inlineStr">
         <is>
           <t>Weighted pull ups 3 x 5 @ 80%, bench 3 x 5 @ 80%.
-Then arms block B: Face pulls 3x15, Bayesian cable curls 3x10-12, hammer curls 3x10-12, cable crunch 3x10
+Then arms block B: Face pulls 3x15, Bayesian cable curls 3x10-12, hammer curls 3x10-12
 Finisher: EMOM 12 min: 1) SkiErg 250 m 2) 25 wall balls 3) 10 burpee broad jumps 4) row 250 m</t>
         </is>
       </c>
@@ -2437,7 +2437,7 @@
       </c>
       <c r="E18" s="49" t="inlineStr">
         <is>
-          <t>Back squat 3 x 5. RDL 3 x 8 @ RPE 7. EMOM 24 min: 1) sled push 15 m at 110% race weight 2) sandbag lunges 25 m, 20 kg 3) farmers 100 m, 2 x 30 kg (above race weight, grip) 4) sled pull 15 m at 110% race weight</t>
+          <t>Back squat 3 x 5. RDL 3 x 8 @ RPE 7. Cable crunch 3x10. EMOM 24 min: 1) sled push 15 m at 110% race weight 2) sandbag lunges 25 m, 20 kg 3) farmers 100 m, 2 x 30 kg (above race weight, grip) 4) sled pull 15 m at 110% race weight</t>
         </is>
       </c>
       <c r="F18" s="49" t="inlineStr">
@@ -2449,7 +2449,7 @@
       <c r="G18" s="49" t="inlineStr">
         <is>
           <t>Weighted pull ups 3 x 5, bench 3 x 5.
-Then arms block B: Face pulls 3x15, Bayesian cable curls 3x10-12, hammer curls 3x10-12, cable crunch 3x10
+Then arms block B: Face pulls 3x15, Bayesian cable curls 3x10-12, hammer curls 3x10-12
 Finisher: EMOM 24 min: 1) SkiErg 250 m 2) 25 wall balls 3) 10 burpee broad jumps 4) row 250 m</t>
         </is>
       </c>
@@ -2489,7 +2489,7 @@
       </c>
       <c r="E19" s="49" t="inlineStr">
         <is>
-          <t>Back squat 3 x 5. RDL 3 x 8 @ RPE 7. EMOM 24 min: 1) sled push 15 m at 110% race weight 2) sandbag lunges 25 m, 20 kg 3) farmers 100 m, 2 x 30 kg (above race weight, grip) 4) sled pull 15 m at 110% race weight</t>
+          <t>Back squat 3 x 5. RDL 3 x 8 @ RPE 7. Cable crunch 3x10. EMOM 24 min: 1) sled push 15 m at 110% race weight 2) sandbag lunges 25 m, 20 kg 3) farmers 100 m, 2 x 30 kg (above race weight, grip) 4) sled pull 15 m at 110% race weight</t>
         </is>
       </c>
       <c r="F19" s="49" t="inlineStr">
@@ -2501,7 +2501,7 @@
       <c r="G19" s="49" t="inlineStr">
         <is>
           <t>Weighted pull ups 3 x 5, bench 3 x 5.
-Then arms block B: Face pulls 3x15, Bayesian cable curls 3x10-12, hammer curls 3x10-12, cable crunch 3x10
+Then arms block B: Face pulls 3x15, Bayesian cable curls 3x10-12, hammer curls 3x10-12
 Finisher: EMOM 24 min: 1) SkiErg 250 m 2) 25 wall balls 3) 10 burpee broad jumps 4) row 250 m</t>
         </is>
       </c>
@@ -2541,7 +2541,7 @@
       </c>
       <c r="E20" s="49" t="inlineStr">
         <is>
-          <t>Back squat 3 x 5. RDL 3 x 8 @ RPE 7. EMOM 16 min (shorter: full sim Saturday): 1) sled push 15 m at 110% race weight 2) sandbag lunges 25 m, 20 kg 3) farmers 100 m, 2 x 30 kg (above race weight, grip) 4) sled pull 15 m at 110% race weight</t>
+          <t>Back squat 3 x 5. RDL 3 x 8 @ RPE 7. Cable crunch 3x10. EMOM 16 min (shorter: full sim Saturday): 1) sled push 15 m at 110% race weight 2) sandbag lunges 25 m, 20 kg 3) farmers 100 m, 2 x 30 kg (above race weight, grip) 4) sled pull 15 m at 110% race weight</t>
         </is>
       </c>
       <c r="F20" s="49" t="inlineStr">
@@ -2553,7 +2553,7 @@
       <c r="G20" s="49" t="inlineStr">
         <is>
           <t>Weighted pull ups 3 x 5, bench 3 x 5.
-Then arms block B: Face pulls 3x15, Bayesian cable curls 3x10-12, hammer curls 3x10-12, cable crunch 3x10
+Then arms block B: Face pulls 3x15, Bayesian cable curls 3x10-12, hammer curls 3x10-12
 Finisher: EMOM 16 min (shorter: full sim Saturday): 1) SkiErg 250 m 2) 25 wall balls 3) 10 burpee broad jumps 4) row 250 m</t>
         </is>
       </c>
@@ -2597,7 +2597,7 @@
       </c>
       <c r="E21" s="49" t="inlineStr">
         <is>
-          <t>Back squat 3 x 5 @ 80%. RDL 3 x 8 @ 80%. EMOM 12 min (3 rounds), normal loads: 1) sled push 15 m at 110% race weight 2) sandbag lunges 25 m, 20 kg 3) farmers 100 m, 2 x 30 kg (above race weight, grip) 4) sled pull 15 m at 110% race weight</t>
+          <t>Back squat 3 x 5 @ 80%. RDL 3 x 8 @ 80%. Cable crunch 3x10. EMOM 12 min (3 rounds), normal loads: 1) sled push 15 m at 110% race weight 2) sandbag lunges 25 m, 20 kg 3) farmers 100 m, 2 x 30 kg (above race weight, grip) 4) sled pull 15 m at 110% race weight</t>
         </is>
       </c>
       <c r="F21" s="49" t="inlineStr">
@@ -2609,7 +2609,7 @@
       <c r="G21" s="49" t="inlineStr">
         <is>
           <t>Weighted pull ups 3 x 5 @ 80%, bench 3 x 5 @ 80%.
-Then arms block B: Face pulls 3x15, Bayesian cable curls 3x10-12, hammer curls 3x10-12, cable crunch 3x10
+Then arms block B: Face pulls 3x15, Bayesian cable curls 3x10-12, hammer curls 3x10-12
 Finisher: EMOM 12 min: 1) SkiErg 250 m 2) 25 wall balls 3) 10 burpee broad jumps 4) row 250 m</t>
         </is>
       </c>
@@ -2653,7 +2653,7 @@
       </c>
       <c r="E22" s="49" t="inlineStr">
         <is>
-          <t>Back squat 3 x 5. RDL 3 x 8 @ RPE 7. EMOM 16 min (shorter: full sim Saturday): 1) sled push 15 m at 110% race weight 2) sandbag lunges 25 m, 20 kg 3) farmers 100 m, 2 x 30 kg (above race weight, grip) 4) sled pull 15 m at 110% race weight</t>
+          <t>Back squat 3 x 5. RDL 3 x 8 @ RPE 7. Cable crunch 3x10. EMOM 16 min (shorter: full sim Saturday): 1) sled push 15 m at 110% race weight 2) sandbag lunges 25 m, 20 kg 3) farmers 100 m, 2 x 30 kg (above race weight, grip) 4) sled pull 15 m at 110% race weight</t>
         </is>
       </c>
       <c r="F22" s="49" t="inlineStr">
@@ -2665,7 +2665,7 @@
       <c r="G22" s="49" t="inlineStr">
         <is>
           <t>Weighted pull ups 3 x 5, bench 3 x 5.
-Then arms block B: Face pulls 3x15, Bayesian cable curls 3x10-12, hammer curls 3x10-12, cable crunch 3x10
+Then arms block B: Face pulls 3x15, Bayesian cable curls 3x10-12, hammer curls 3x10-12
 Finisher: EMOM 16 min (shorter: full sim Saturday): 1) SkiErg 250 m 2) 25 wall balls 3) 10 burpee broad jumps 4) row 250 m</t>
         </is>
       </c>
@@ -2705,7 +2705,7 @@
       </c>
       <c r="E23" s="49" t="inlineStr">
         <is>
-          <t>Squat 3 x 3. EMOM 20 min at race weight and race effort: 1) sled push 25 m 2) lunges 25 m 3) farmers 100 m 4) sled pull 25 m</t>
+          <t>Squat 3 x 3. Cable crunch 3x10. EMOM 20 min at race weight and race effort: 1) sled push 25 m 2) lunges 25 m 3) farmers 100 m 4) sled pull 25 m</t>
         </is>
       </c>
       <c r="F23" s="49" t="inlineStr">
@@ -2717,7 +2717,7 @@
       <c r="G23" s="49" t="inlineStr">
         <is>
           <t>Pull ups 3 x 5, press 3 x 5.
-Then arms block B: Face pulls 3x15, Bayesian cable curls 3x10-12, hammer curls 3x10-12, cable crunch 3x10
+Then arms block B: Face pulls 3x15, Bayesian cable curls 3x10-12, hammer curls 3x10-12
 Finisher: EMOM 20 min at race effort: 1) SkiErg 250 m 2) 25 wall balls 3) 10 burpee broad jumps 4) row 250 m</t>
         </is>
       </c>
@@ -2757,7 +2757,7 @@
       </c>
       <c r="E24" s="49" t="inlineStr">
         <is>
-          <t>Squat 3 x 3. EMOM 20 min at race weight and race effort: 1) sled push 25 m 2) lunges 25 m 3) farmers 100 m 4) sled pull 25 m</t>
+          <t>Squat 3 x 3. Cable crunch 3x10. EMOM 20 min at race weight and race effort: 1) sled push 25 m 2) lunges 25 m 3) farmers 100 m 4) sled pull 25 m</t>
         </is>
       </c>
       <c r="F24" s="49" t="inlineStr">
@@ -2769,7 +2769,7 @@
       <c r="G24" s="49" t="inlineStr">
         <is>
           <t>Pull ups 3 x 5, press 3 x 5.
-Then arms block B: Face pulls 3x15, Bayesian cable curls 3x10-12, hammer curls 3x10-12, cable crunch 3x10
+Then arms block B: Face pulls 3x15, Bayesian cable curls 3x10-12, hammer curls 3x10-12
 Finisher: EMOM 20 min at race effort: 1) SkiErg 250 m 2) 25 wall balls 3) 10 burpee broad jumps 4) row 250 m</t>
         </is>
       </c>

</xml_diff>

<commit_message>
v121: run km target = planned runs only (no warm ups)
Fred (Oct 24) did every week 4 session and the km bar showed 6.4 of 7,
because the targets included an allowance for warm ups he does not log.
PLAN runKm for all 27 weeks is now Tuesday's run (reps x distance, or the
tempo/easy km) + the sim runs + the Sunday zone 2 run (week 4 11.4, so
6.4 without Sunday). Excel column J updated. Replaces the warm up
allowance and the v107 deload +1/+2 bumps. Tests: kmbar, deload, sunrun,
header updated.

Coach impact: PROMPT.md says runKm is the planned run distance only.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_017ty1gcaEfLM16MJZGfipS3
</commit_message>
<xml_diff>
--- a/plan/HYROX_Brisbane_2027_Plan.xlsx
+++ b/plan/HYROX_Brisbane_2027_Plan.xlsx
@@ -1543,7 +1543,7 @@
       </c>
       <c r="J1" s="48" t="inlineStr">
         <is>
-          <t>Run km target</t>
+          <t>Run km target (planned runs only, no warm ups)</t>
         </is>
       </c>
       <c r="K1" s="48" t="inlineStr">
@@ -1604,7 +1604,7 @@
         </is>
       </c>
       <c r="J2" s="49" t="n">
-        <v>8</v>
+        <v>4.4</v>
       </c>
       <c r="K2" s="58" t="inlineStr">
         <is>
@@ -1660,7 +1660,7 @@
         </is>
       </c>
       <c r="J3" s="49" t="n">
-        <v>9</v>
+        <v>5.2</v>
       </c>
       <c r="K3" s="58" t="n"/>
       <c r="L3" s="59" t="n"/>
@@ -1712,7 +1712,7 @@
         </is>
       </c>
       <c r="J4" s="49" t="n">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="K4" s="58" t="n"/>
       <c r="L4" s="59" t="n"/>
@@ -1764,7 +1764,7 @@
         </is>
       </c>
       <c r="J5" s="49" t="n">
-        <v>12</v>
+        <v>11.4</v>
       </c>
       <c r="K5" s="58" t="n"/>
       <c r="L5" s="59" t="n"/>
@@ -1816,7 +1816,7 @@
         </is>
       </c>
       <c r="J6" s="49" t="n">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="K6" s="58" t="n"/>
       <c r="L6" s="59" t="n"/>
@@ -1868,7 +1868,7 @@
         </is>
       </c>
       <c r="J7" s="49" t="n">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="K7" s="58" t="n"/>
       <c r="L7" s="59" t="inlineStr">
@@ -1924,7 +1924,7 @@
         </is>
       </c>
       <c r="J8" s="49" t="n">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="K8" s="58" t="n"/>
       <c r="L8" s="59" t="n"/>
@@ -1976,7 +1976,7 @@
         </is>
       </c>
       <c r="J9" s="49" t="n">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="K9" s="58" t="n"/>
       <c r="L9" s="59" t="inlineStr">
@@ -2032,7 +2032,7 @@
         </is>
       </c>
       <c r="J10" s="49" t="n">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="K10" s="58" t="n"/>
       <c r="L10" s="59" t="inlineStr">
@@ -2088,7 +2088,7 @@
         </is>
       </c>
       <c r="J11" s="49" t="n">
-        <v>18</v>
+        <v>13</v>
       </c>
       <c r="K11" s="58" t="n"/>
       <c r="L11" s="59" t="n"/>
@@ -2140,7 +2140,7 @@
         </is>
       </c>
       <c r="J12" s="49" t="n">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="K12" s="58" t="n"/>
       <c r="L12" s="59" t="inlineStr">
@@ -2196,7 +2196,7 @@
         </is>
       </c>
       <c r="J13" s="49" t="n">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="K13" s="58" t="n"/>
       <c r="L13" s="59" t="n"/>
@@ -2248,7 +2248,7 @@
         </is>
       </c>
       <c r="J14" s="49" t="n">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="K14" s="58" t="n"/>
       <c r="L14" s="59" t="inlineStr">
@@ -2304,7 +2304,7 @@
         </is>
       </c>
       <c r="J15" s="49" t="n">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="K15" s="58" t="n"/>
       <c r="L15" s="59" t="n"/>
@@ -2356,7 +2356,7 @@
         </is>
       </c>
       <c r="J16" s="49" t="n">
-        <v>20</v>
+        <v>14</v>
       </c>
       <c r="K16" s="58" t="n"/>
       <c r="L16" s="59" t="n"/>
@@ -2408,7 +2408,7 @@
         </is>
       </c>
       <c r="J17" s="49" t="n">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="K17" s="58" t="n"/>
       <c r="L17" s="59" t="inlineStr">
@@ -2464,7 +2464,7 @@
         </is>
       </c>
       <c r="J18" s="49" t="n">
-        <v>21</v>
+        <v>17</v>
       </c>
       <c r="K18" s="58" t="n"/>
       <c r="L18" s="59" t="n"/>
@@ -2516,7 +2516,7 @@
         </is>
       </c>
       <c r="J19" s="49" t="n">
-        <v>22</v>
+        <v>17</v>
       </c>
       <c r="K19" s="58" t="n"/>
       <c r="L19" s="59" t="n"/>
@@ -2568,7 +2568,7 @@
         </is>
       </c>
       <c r="J20" s="49" t="n">
-        <v>23</v>
+        <v>18</v>
       </c>
       <c r="K20" s="58" t="n"/>
       <c r="L20" s="59" t="inlineStr">
@@ -2624,7 +2624,7 @@
         </is>
       </c>
       <c r="J21" s="49" t="n">
-        <v>18</v>
+        <v>13</v>
       </c>
       <c r="K21" s="58" t="n"/>
       <c r="L21" s="59" t="inlineStr">
@@ -2680,7 +2680,7 @@
         </is>
       </c>
       <c r="J22" s="49" t="n">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="K22" s="58" t="n"/>
       <c r="L22" s="59" t="n"/>
@@ -2732,7 +2732,7 @@
         </is>
       </c>
       <c r="J23" s="49" t="n">
-        <v>24</v>
+        <v>15</v>
       </c>
       <c r="K23" s="58" t="n"/>
       <c r="L23" s="59" t="n"/>
@@ -2784,7 +2784,7 @@
         </is>
       </c>
       <c r="J24" s="49" t="n">
-        <v>25</v>
+        <v>17</v>
       </c>
       <c r="K24" s="58" t="n"/>
       <c r="L24" s="59" t="n"/>
@@ -2836,7 +2836,7 @@
         </is>
       </c>
       <c r="J25" s="49" t="n">
-        <v>25</v>
+        <v>18</v>
       </c>
       <c r="K25" s="58" t="n"/>
       <c r="L25" s="59" t="inlineStr">
@@ -2892,7 +2892,7 @@
         </is>
       </c>
       <c r="J26" s="49" t="n">
-        <v>18</v>
+        <v>13</v>
       </c>
       <c r="K26" s="58" t="n"/>
       <c r="L26" s="59" t="n"/>
@@ -2942,7 +2942,7 @@
         </is>
       </c>
       <c r="J27" s="49" t="n">
-        <v>10</v>
+        <v>4</v>
       </c>
       <c r="K27" s="58" t="n"/>
       <c r="L27" s="59" t="inlineStr">
@@ -2995,7 +2995,7 @@
         </is>
       </c>
       <c r="J28" s="49" t="n">
-        <v>6</v>
+        <v>11</v>
       </c>
       <c r="K28" s="58" t="n"/>
       <c r="L28" s="59" t="inlineStr">

</xml_diff>

<commit_message>
Excel: Overview note says only the technique sets are Fred only
Coach impact: none.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_017ty1gcaEfLM16MJZGfipS3
</commit_message>
<xml_diff>
--- a/plan/HYROX_Brisbane_2027_Plan.xlsx
+++ b/plan/HYROX_Brisbane_2027_Plan.xlsx
@@ -702,7 +702,6 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
     <row r="3" ht="15" customHeight="1" s="39">
       <c r="A3" s="41" t="inlineStr">
         <is>
@@ -802,7 +801,6 @@
         </is>
       </c>
     </row>
-    <row r="11"/>
     <row r="12" ht="15" customHeight="1" s="39">
       <c r="A12" s="47" t="inlineStr">
         <is>
@@ -824,7 +822,6 @@
         </is>
       </c>
     </row>
-    <row r="15"/>
     <row r="16" ht="15" customHeight="1" s="39">
       <c r="A16" s="47" t="inlineStr">
         <is>
@@ -1066,8 +1063,6 @@
         </is>
       </c>
     </row>
-    <row r="27"/>
-    <row r="28"/>
     <row r="29" ht="15" customHeight="1" s="39">
       <c r="A29" s="47" t="inlineStr">
         <is>
@@ -1264,7 +1259,6 @@
         </is>
       </c>
     </row>
-    <row r="37"/>
     <row r="38" ht="15" customHeight="1" s="39">
       <c r="A38" s="47" t="inlineStr">
         <is>
@@ -1371,7 +1365,6 @@
         </is>
       </c>
     </row>
-    <row r="47"/>
     <row r="48" ht="15" customHeight="1" s="39">
       <c r="A48" s="47" t="inlineStr">
         <is>
@@ -1474,9 +1467,9 @@
       <c r="A62" s="42" t="n"/>
     </row>
     <row r="63">
-      <c r="A63" t="inlineStr">
-        <is>
-          <t>Fred only (Oct 31): wall ball technique 2 x 10 on Fridays weeks 6 to 21; weeks 15 to 21 EMOM wall balls with a 9 kg (20 lb) ball and Monday sandbag lunges at 25 kg. Will and Grady keep the base plan in the app.</t>
+      <c r="A63" s="38" t="inlineStr">
+        <is>
+          <t>Oct 31: Fridays weeks 6 to 21 add wall ball technique 2 x 10 (Fred only). Weeks 15 to 21 for everyone: EMOM wall balls with a 9 kg (20 lb) ball and Monday sandbag lunges at 25 kg.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
v126: week 6 sim runs are full 1 km (8 x 1 km + station at half volume)
Fred and Will asked on Oct 30 and confirmed Oct 31 for the Nov 7 sim: keep stations at half volume, run full 1 km laps. Applies to every athlete.

- PLAN week 6 sat: 8 x (1 km run + station at half volume); runKm 14 to 18 (core target 13 without Sunday).
- Excel week 6 columns H and J updated.
- tests: kmbar runKm list, adaptive test override now uses a full volume variant. Full suite green.

Coach impact: PROMPT.md Nashville line says week 6 is 8 x 1 km now. The sim report will flag the lap length change vs the previous sim and compare run pace per km.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_017ty1gcaEfLM16MJZGfipS3
</commit_message>
<xml_diff>
--- a/plan/HYROX_Brisbane_2027_Plan.xlsx
+++ b/plan/HYROX_Brisbane_2027_Plan.xlsx
@@ -1867,7 +1867,7 @@
       </c>
       <c r="H7" s="49" t="inlineStr">
         <is>
-          <t>Half sim, 75%, half volume, all 8 stations in race order: 8 x (500 m run + station at half volume)</t>
+          <t>Half sim, 75%, half volume, all 8 stations in race order: 8 x (1 km run + station at half volume)</t>
         </is>
       </c>
       <c r="I7" s="49" t="inlineStr">
@@ -1876,7 +1876,7 @@
         </is>
       </c>
       <c r="J7" s="49" t="n">
-        <v>14</v>
+        <v>18</v>
       </c>
       <c r="K7" s="58" t="n"/>
       <c r="L7" s="59" t="inlineStr">

</xml_diff>